<commit_message>
Update WS1-Terms blank labels with corrected cognitive task names
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -942,10 +942,10 @@
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B17:E17"/>
     <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B23:E23"/>
     <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B17:E17"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B16:E16"/>
@@ -3364,67 +3364,67 @@
       <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Blank 1
-Label name</t>
+Target Label</t>
         </is>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
           <t>Blank 2
-Object name</t>
+Data Object</t>
         </is>
       </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Blank 3
-Feature name</t>
+Feature Name</t>
         </is>
       </c>
       <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Blank 4
-Feature value</t>
+Feature Value</t>
         </is>
       </c>
       <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Blank 5
-Object definition</t>
+Data Instance</t>
         </is>
       </c>
       <c r="H3" s="24" t="inlineStr">
         <is>
           <t>Blank 6
-Object example</t>
+Specific Object</t>
         </is>
       </c>
       <c r="I3" s="24" t="inlineStr">
         <is>
           <t>Blank 7
-Feature term</t>
+Feature Variable</t>
         </is>
       </c>
       <c r="J3" s="24" t="inlineStr">
         <is>
           <t>Blank 8
-Feature count</t>
+Feature Count</t>
         </is>
       </c>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>Blank 9
-Feature list</t>
+Feature List</t>
         </is>
       </c>
       <c r="L3" s="24" t="inlineStr">
         <is>
           <t>Blank 10
-Object example 2</t>
+Instance Name</t>
         </is>
       </c>
       <c r="M3" s="24" t="inlineStr">
         <is>
           <t>Blank 11
-Label term</t>
+Assigned Label</t>
         </is>
       </c>
       <c r="N3" s="24" t="inlineStr">

</xml_diff>

<commit_message>
WS3 row 54: write 8 task descriptions in order; remove descriptions from row 3 all sheets
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -226,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -360,6 +360,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1376,42 +1382,38 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="28" t="inlineStr"/>
-      <c r="H5" s="28" t="inlineStr"/>
-      <c r="I5" s="28" t="inlineStr"/>
-      <c r="J5" s="28" t="inlineStr"/>
-      <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="28" t="inlineStr"/>
-      <c r="M5" s="28" t="inlineStr"/>
-      <c r="N5" s="28" t="inlineStr"/>
-      <c r="O5" s="28" t="inlineStr"/>
-      <c r="P5" s="28" t="inlineStr"/>
-      <c r="Q5" s="28" t="inlineStr"/>
-      <c r="R5" s="28" t="inlineStr"/>
-      <c r="S5" s="28" t="inlineStr"/>
-      <c r="T5" s="28" t="inlineStr"/>
-      <c r="U5" s="28" t="inlineStr"/>
-      <c r="V5" s="28" t="inlineStr"/>
-      <c r="W5" s="28" t="inlineStr"/>
-      <c r="X5" s="28" t="inlineStr"/>
-      <c r="Y5" s="28" t="inlineStr"/>
-      <c r="Z5" s="28" t="inlineStr"/>
-      <c r="AA5" s="29" t="inlineStr"/>
-      <c r="AB5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="47" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="47" t="n"/>
+      <c r="K5" s="47" t="n"/>
+      <c r="L5" s="47" t="n"/>
+      <c r="M5" s="47" t="n"/>
+      <c r="N5" s="47" t="n"/>
+      <c r="O5" s="47" t="n"/>
+      <c r="P5" s="47" t="n"/>
+      <c r="Q5" s="47" t="n"/>
+      <c r="R5" s="47" t="n"/>
+      <c r="S5" s="47" t="n"/>
+      <c r="T5" s="47" t="n"/>
+      <c r="U5" s="47" t="n"/>
+      <c r="V5" s="47" t="n"/>
+      <c r="W5" s="47" t="n"/>
+      <c r="X5" s="47" t="n"/>
+      <c r="Y5" s="47" t="n"/>
+      <c r="Z5" s="47" t="n"/>
+      <c r="AA5" s="47" t="n"/>
+      <c r="AB5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -2519,42 +2521,38 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="28" t="inlineStr"/>
-      <c r="H36" s="28" t="inlineStr"/>
-      <c r="I36" s="28" t="inlineStr"/>
-      <c r="J36" s="28" t="inlineStr"/>
-      <c r="K36" s="28" t="inlineStr"/>
-      <c r="L36" s="28" t="inlineStr"/>
-      <c r="M36" s="28" t="inlineStr"/>
-      <c r="N36" s="28" t="inlineStr"/>
-      <c r="O36" s="28" t="inlineStr"/>
-      <c r="P36" s="28" t="inlineStr"/>
-      <c r="Q36" s="28" t="inlineStr"/>
-      <c r="R36" s="28" t="inlineStr"/>
-      <c r="S36" s="28" t="inlineStr"/>
-      <c r="T36" s="28" t="inlineStr"/>
-      <c r="U36" s="28" t="inlineStr"/>
-      <c r="V36" s="28" t="inlineStr"/>
-      <c r="W36" s="28" t="inlineStr"/>
-      <c r="X36" s="28" t="inlineStr"/>
-      <c r="Y36" s="28" t="inlineStr"/>
-      <c r="Z36" s="28" t="inlineStr"/>
-      <c r="AA36" s="29" t="inlineStr"/>
-      <c r="AB36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="n"/>
+      <c r="K36" s="47" t="n"/>
+      <c r="L36" s="47" t="n"/>
+      <c r="M36" s="47" t="n"/>
+      <c r="N36" s="47" t="n"/>
+      <c r="O36" s="47" t="n"/>
+      <c r="P36" s="47" t="n"/>
+      <c r="Q36" s="47" t="n"/>
+      <c r="R36" s="47" t="n"/>
+      <c r="S36" s="47" t="n"/>
+      <c r="T36" s="47" t="n"/>
+      <c r="U36" s="47" t="n"/>
+      <c r="V36" s="47" t="n"/>
+      <c r="W36" s="47" t="n"/>
+      <c r="X36" s="47" t="n"/>
+      <c r="Y36" s="47" t="n"/>
+      <c r="Z36" s="47" t="n"/>
+      <c r="AA36" s="47" t="n"/>
+      <c r="AB36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -3126,7 +3124,6 @@
       <c r="AA51" s="29" t="inlineStr"/>
       <c r="AB51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -3414,78 +3411,67 @@
       <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Blank 1
-Target Label
-Determining the final classification result (e.g., 'not recommendable')</t>
+Target Label</t>
         </is>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
           <t>Blank 2
-Data Object
-Recognizing the fundamental data entity or item (e.g., 'Hazelnut Wafer')</t>
+Data Object</t>
         </is>
       </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Blank 3
-Feature Name
-Identifying the name of the independent variable (e.g., 'Fat')</t>
+Feature Name</t>
         </is>
       </c>
       <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Blank 4
-Feature Value
-Extracting the specific quantitative measurement for an attribute (e.g., '31.9 g')</t>
+Feature Value</t>
         </is>
       </c>
       <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Blank 5
-Data Instance
-Comprehending that an item acts as a single row or data point in a dataset (e.g., 'Individual foods are called objects...')</t>
+Data Instance</t>
         </is>
       </c>
       <c r="H3" s="24" t="inlineStr">
         <is>
           <t>Blank 6
-Specific Object
-Mapping a concrete, real-world example to the concept of a data object (e.g., 'A hazelnut wafer is an object')</t>
+Specific Object</t>
         </is>
       </c>
       <c r="I3" s="24" t="inlineStr">
         <is>
           <t>Blank 7
-Feature Variable
-Understanding the structural attributes (columns) that describe the data (e.g., 'features are located in the left column')</t>
+Feature Variable</t>
         </is>
       </c>
       <c r="J3" s="24" t="inlineStr">
         <is>
           <t>Blank 8
-Feature Count
-Calculating the dimensionality or total number of variables in the dataset (e.g., 'there are 7 features')</t>
+Feature Count</t>
         </is>
       </c>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>Blank 9
-Feature List
-Enumerating all the independent variables that can be extracted (e.g., 'Energy, Fat, Saturated Fat...')</t>
+Feature List</t>
         </is>
       </c>
       <c r="L3" s="24" t="inlineStr">
         <is>
           <t>Blank 10
-Instance Name
-Associating a specific data value (like 31.9 g) back to the specific object it belongs to (e.g., 'Hazelnut Wafer contains 31.9 g of fat')</t>
+Instance Name</t>
         </is>
       </c>
       <c r="M3" s="24" t="inlineStr">
         <is>
           <t>Blank 11
-Assigned Label
-Grasping that the target variable serves as the final decision or output for that specific item (e.g., 'given the note not recommendable as a label...')</t>
+Assigned Label</t>
         </is>
       </c>
       <c r="N3" s="24" t="inlineStr">
@@ -3507,29 +3493,25 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="28" t="inlineStr"/>
-      <c r="H5" s="28" t="inlineStr"/>
-      <c r="I5" s="28" t="inlineStr"/>
-      <c r="J5" s="28" t="inlineStr"/>
-      <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="28" t="inlineStr"/>
-      <c r="M5" s="28" t="inlineStr"/>
-      <c r="N5" s="29" t="inlineStr"/>
-      <c r="O5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="47" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="47" t="n"/>
+      <c r="K5" s="47" t="n"/>
+      <c r="L5" s="47" t="n"/>
+      <c r="M5" s="47" t="n"/>
+      <c r="N5" s="47" t="n"/>
+      <c r="O5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -4260,29 +4242,25 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="28" t="inlineStr"/>
-      <c r="H36" s="28" t="inlineStr"/>
-      <c r="I36" s="28" t="inlineStr"/>
-      <c r="J36" s="28" t="inlineStr"/>
-      <c r="K36" s="28" t="inlineStr"/>
-      <c r="L36" s="28" t="inlineStr"/>
-      <c r="M36" s="28" t="inlineStr"/>
-      <c r="N36" s="29" t="inlineStr"/>
-      <c r="O36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="n"/>
+      <c r="K36" s="47" t="n"/>
+      <c r="L36" s="47" t="n"/>
+      <c r="M36" s="47" t="n"/>
+      <c r="N36" s="47" t="n"/>
+      <c r="O36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -4659,7 +4637,6 @@
       <c r="N51" s="29" t="inlineStr"/>
       <c r="O51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -4764,7 +4741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4880,22 +4857,18 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="29" t="inlineStr"/>
-      <c r="H5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -5423,22 +5396,18 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="29" t="inlineStr"/>
-      <c r="H36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -5710,7 +5679,6 @@
       <c r="G51" s="29" t="inlineStr"/>
       <c r="H51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -5725,34 +5693,44 @@
         </is>
       </c>
       <c r="B54" s="35" t="inlineStr"/>
-      <c r="C54" s="36" t="inlineStr">
-        <is>
-          <t>Classifies popcorn as recommended (fat &lt;= 8g) AND gives correct justification</t>
-        </is>
-      </c>
-      <c r="D54" s="36" t="inlineStr">
-        <is>
-          <t>Classifies apple as recommended AND gives correct justification referencing fat value</t>
-        </is>
-      </c>
-      <c r="E54" s="36" t="inlineStr">
-        <is>
-          <t>Classifies french fries as not recommended (fat &gt; 8g) AND gives correct justification</t>
-        </is>
-      </c>
-      <c r="F54" s="36" t="inlineStr">
-        <is>
-          <t>Writes own threshold for the Energy variable with correct &lt;= / &gt; notation in the diagram</t>
-        </is>
-      </c>
-      <c r="G54" s="36" t="inlineStr">
-        <is>
-          <t>Overall AI-CFT level for WS3 as a whole</t>
-        </is>
-      </c>
-      <c r="H54" s="36" t="inlineStr">
-        <is>
-          <t>Free notes</t>
+      <c r="C54" s="50" t="inlineStr">
+        <is>
+          <t>Instance Classification (Popcorn): Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
+        </is>
+      </c>
+      <c r="D54" s="50" t="inlineStr">
+        <is>
+          <t>Rule Verification (Popcorn): Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "23.0 &gt; 8.0").</t>
+        </is>
+      </c>
+      <c r="E54" s="50" t="inlineStr">
+        <is>
+          <t>Instance Classification (Apple): Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilebilir").</t>
+        </is>
+      </c>
+      <c r="F54" s="50" t="inlineStr">
+        <is>
+          <t>Rule Verification (Apple): Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "8.0 &gt; 0.2").</t>
+        </is>
+      </c>
+      <c r="G54" s="50" t="inlineStr">
+        <is>
+          <t>Instance Classification (French Fries): Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
+        </is>
+      </c>
+      <c r="H54" s="50" t="inlineStr">
+        <is>
+          <t>Rule Verification (French Fries): Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "14.0 &gt; 8.0").</t>
+        </is>
+      </c>
+      <c r="I54" s="45" t="inlineStr">
+        <is>
+          <t>Left Branching Condition: Establishing the mathematical boundary expression (≤) for a split node based on the data distribution of the feature (e.g., ≤ 71 kcal).</t>
+        </is>
+      </c>
+      <c r="J54" s="45" t="inlineStr">
+        <is>
+          <t>Right Branching Condition: Establishing the corresponding inverse mathematical expression (&gt;) for a split node to partition the remaining instances in the dataset (e.g., &gt; 71 kcal).</t>
         </is>
       </c>
     </row>
@@ -5896,22 +5874,18 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="29" t="inlineStr"/>
-      <c r="H5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -6439,22 +6413,18 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="29" t="inlineStr"/>
-      <c r="H36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -6726,7 +6696,6 @@
       <c r="G51" s="29" t="inlineStr"/>
       <c r="H51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -6948,25 +6917,21 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="28" t="inlineStr"/>
-      <c r="H5" s="28" t="inlineStr"/>
-      <c r="I5" s="28" t="inlineStr"/>
-      <c r="J5" s="29" t="inlineStr"/>
-      <c r="K5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="47" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="47" t="n"/>
+      <c r="K5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -7581,25 +7546,21 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="28" t="inlineStr"/>
-      <c r="H36" s="28" t="inlineStr"/>
-      <c r="I36" s="28" t="inlineStr"/>
-      <c r="J36" s="29" t="inlineStr"/>
-      <c r="K36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="n"/>
+      <c r="K36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -7916,7 +7877,6 @@
       <c r="J51" s="29" t="inlineStr"/>
       <c r="K51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -8153,25 +8113,21 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="28" t="inlineStr"/>
-      <c r="H5" s="28" t="inlineStr"/>
-      <c r="I5" s="28" t="inlineStr"/>
-      <c r="J5" s="29" t="inlineStr"/>
-      <c r="K5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="47" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="47" t="n"/>
+      <c r="K5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -8786,25 +8742,21 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="28" t="inlineStr"/>
-      <c r="H36" s="28" t="inlineStr"/>
-      <c r="I36" s="28" t="inlineStr"/>
-      <c r="J36" s="29" t="inlineStr"/>
-      <c r="K36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="n"/>
+      <c r="K36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -9121,7 +9073,6 @@
       <c r="J51" s="29" t="inlineStr"/>
       <c r="K51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -9358,25 +9309,21 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="28" t="inlineStr"/>
-      <c r="H5" s="28" t="inlineStr"/>
-      <c r="I5" s="28" t="inlineStr"/>
-      <c r="J5" s="29" t="inlineStr"/>
-      <c r="K5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="47" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="47" t="n"/>
+      <c r="K5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -9991,25 +9938,21 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="28" t="inlineStr"/>
-      <c r="H36" s="28" t="inlineStr"/>
-      <c r="I36" s="28" t="inlineStr"/>
-      <c r="J36" s="29" t="inlineStr"/>
-      <c r="K36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="n"/>
+      <c r="K36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -10326,7 +10269,6 @@
       <c r="J51" s="29" t="inlineStr"/>
       <c r="K51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -10515,21 +10457,17 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="29" t="inlineStr"/>
-      <c r="G5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -11028,21 +10966,17 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="29" t="inlineStr"/>
-      <c r="G36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -11299,7 +11233,6 @@
       <c r="F51" s="29" t="inlineStr"/>
       <c r="G51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>
@@ -11516,25 +11449,21 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="28" t="inlineStr"/>
-      <c r="H5" s="28" t="inlineStr"/>
-      <c r="I5" s="28" t="inlineStr"/>
-      <c r="J5" s="29" t="inlineStr"/>
-      <c r="K5" s="30" t="inlineStr"/>
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="47" t="n"/>
+      <c r="H5" s="47" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="47" t="n"/>
+      <c r="K5" s="48" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -12149,25 +12078,21 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr"/>
-      <c r="D36" s="28" t="inlineStr"/>
-      <c r="E36" s="28" t="inlineStr"/>
-      <c r="F36" s="28" t="inlineStr"/>
-      <c r="G36" s="28" t="inlineStr"/>
-      <c r="H36" s="28" t="inlineStr"/>
-      <c r="I36" s="28" t="inlineStr"/>
-      <c r="J36" s="29" t="inlineStr"/>
-      <c r="K36" s="30" t="inlineStr"/>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="47" t="n"/>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="n"/>
+      <c r="K36" s="48" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
@@ -12484,7 +12409,6 @@
       <c r="J51" s="29" t="inlineStr"/>
       <c r="K51" s="30" t="inlineStr"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
WS3: titles to row 3, descriptions to row 54
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,6 +113,16 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -225,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -364,6 +374,18 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4789,38 +4811,44 @@
           <t>Student Name</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Task 1
-Popcorn</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
-        <is>
-          <t>Task 2
-Apple</t>
-        </is>
-      </c>
-      <c r="E3" s="16" t="inlineStr">
-        <is>
-          <t>Task 3
-Fries</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
-        <is>
-          <t>Task 4
-Own energy threshold</t>
-        </is>
-      </c>
-      <c r="G3" s="16" t="inlineStr">
-        <is>
-          <t>Overall WS3</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="inlineStr">
-        <is>
-          <t>Notes WS3</t>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>Instance Classification (Popcorn)</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>Rule Verification (Popcorn)</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>Instance Classification (Apple)</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>Rule Verification (Apple)</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>Instance Classification (French Fries)</t>
+        </is>
+      </c>
+      <c r="H3" s="52" t="inlineStr">
+        <is>
+          <t>Rule Verification (French Fries)</t>
+        </is>
+      </c>
+      <c r="I3" s="53" t="inlineStr">
+        <is>
+          <t>Left Branching Condition</t>
+        </is>
+      </c>
+      <c r="J3" s="53" t="inlineStr">
+        <is>
+          <t>Right Branching Condition</t>
         </is>
       </c>
     </row>
@@ -5668,52 +5696,44 @@
         </is>
       </c>
       <c r="B54" s="25" t="n"/>
-      <c r="C54" s="50" t="inlineStr">
-        <is>
-          <t>Instance Classification (Popcorn)
-Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
-        </is>
-      </c>
-      <c r="D54" s="50" t="inlineStr">
-        <is>
-          <t>Rule Verification (Popcorn)
-Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "23.0 &gt; 8.0").</t>
-        </is>
-      </c>
-      <c r="E54" s="50" t="inlineStr">
-        <is>
-          <t>Instance Classification (Apple)
-Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilebilir").</t>
-        </is>
-      </c>
-      <c r="F54" s="50" t="inlineStr">
-        <is>
-          <t>Rule Verification (Apple)
-Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "8.0 &gt; 0.2").</t>
-        </is>
-      </c>
-      <c r="G54" s="50" t="inlineStr">
-        <is>
-          <t>Instance Classification (French Fries)
-Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
-        </is>
-      </c>
-      <c r="H54" s="50" t="inlineStr">
-        <is>
-          <t>Rule Verification (French Fries)
-Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "14.0 &gt; 8.0").</t>
-        </is>
-      </c>
-      <c r="I54" s="51" t="inlineStr">
-        <is>
-          <t>Left Branching Condition
-Establishing the mathematical boundary expression (≤) for a split node based on the data distribution of the feature (e.g., ≤ 71 kcal).</t>
-        </is>
-      </c>
-      <c r="J54" s="51" t="inlineStr">
-        <is>
-          <t>Right Branching Condition
-Establishing the corresponding inverse mathematical expression (&gt;) for a split node to partition the remaining instances in the dataset (e.g., &gt; 71 kcal).</t>
+      <c r="C54" s="54" t="inlineStr">
+        <is>
+          <t>Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
+        </is>
+      </c>
+      <c r="D54" s="54" t="inlineStr">
+        <is>
+          <t>Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "23.0 &gt; 8.0").</t>
+        </is>
+      </c>
+      <c r="E54" s="54" t="inlineStr">
+        <is>
+          <t>Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilebilir").</t>
+        </is>
+      </c>
+      <c r="F54" s="54" t="inlineStr">
+        <is>
+          <t>Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "8.0 &gt; 0.2").</t>
+        </is>
+      </c>
+      <c r="G54" s="54" t="inlineStr">
+        <is>
+          <t>Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
+        </is>
+      </c>
+      <c r="H54" s="54" t="inlineStr">
+        <is>
+          <t>Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "14.0 &gt; 8.0").</t>
+        </is>
+      </c>
+      <c r="I54" s="55" t="inlineStr">
+        <is>
+          <t>Establishing the mathematical boundary expression (≤) for a split node based on the data distribution of the feature (e.g., ≤ 71 kcal).</t>
+        </is>
+      </c>
+      <c r="J54" s="55" t="inlineStr">
+        <is>
+          <t>Establishing the corresponding inverse mathematical expression (&gt;) for a split node to partition the remaining instances in the dataset (e.g., &gt; 71 kcal).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WS3 row 3: add Blank numbering, white font
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -124,6 +124,12 @@
       <name val="Calibri"/>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="11">
@@ -235,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -386,6 +392,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4811,44 +4823,52 @@
           <t>Student Name</t>
         </is>
       </c>
-      <c r="C3" s="52" t="inlineStr">
-        <is>
-          <t>Instance Classification (Popcorn)</t>
-        </is>
-      </c>
-      <c r="D3" s="52" t="inlineStr">
-        <is>
-          <t>Rule Verification (Popcorn)</t>
-        </is>
-      </c>
-      <c r="E3" s="52" t="inlineStr">
-        <is>
-          <t>Instance Classification (Apple)</t>
-        </is>
-      </c>
-      <c r="F3" s="52" t="inlineStr">
-        <is>
-          <t>Rule Verification (Apple)</t>
-        </is>
-      </c>
-      <c r="G3" s="52" t="inlineStr">
-        <is>
-          <t>Instance Classification (French Fries)</t>
-        </is>
-      </c>
-      <c r="H3" s="52" t="inlineStr">
-        <is>
-          <t>Rule Verification (French Fries)</t>
-        </is>
-      </c>
-      <c r="I3" s="53" t="inlineStr">
-        <is>
-          <t>Left Branching Condition</t>
-        </is>
-      </c>
-      <c r="J3" s="53" t="inlineStr">
-        <is>
-          <t>Right Branching Condition</t>
+      <c r="C3" s="56" t="inlineStr">
+        <is>
+          <t>Blank 1
+Instance Classification (Popcorn)</t>
+        </is>
+      </c>
+      <c r="D3" s="56" t="inlineStr">
+        <is>
+          <t>Blank 2
+Rule Verification (Popcorn)</t>
+        </is>
+      </c>
+      <c r="E3" s="56" t="inlineStr">
+        <is>
+          <t>Blank 3
+Instance Classification (Apple)</t>
+        </is>
+      </c>
+      <c r="F3" s="56" t="inlineStr">
+        <is>
+          <t>Blank 4
+Rule Verification (Apple)</t>
+        </is>
+      </c>
+      <c r="G3" s="56" t="inlineStr">
+        <is>
+          <t>Blank 5
+Instance Classification (French Fries)</t>
+        </is>
+      </c>
+      <c r="H3" s="56" t="inlineStr">
+        <is>
+          <t>Blank 6
+Rule Verification (French Fries)</t>
+        </is>
+      </c>
+      <c r="I3" s="57" t="inlineStr">
+        <is>
+          <t>Blank 7
+Left Branching Condition</t>
+        </is>
+      </c>
+      <c r="J3" s="57" t="inlineStr">
+        <is>
+          <t>Blank 8
+Right Branching Condition</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WS3: restore Overall/Notes at cols 11-12, fix AI-CFT levels for blanks 5-8
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -241,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -398,6 +398,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4753,7 +4756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="36" min="1" max="1"/>
@@ -4801,12 +4804,32 @@
           <t>Deepen</t>
         </is>
       </c>
-      <c r="G2" s="29" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>Acquire</t>
+        </is>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>Acquire</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>Acquire</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>Acquire</t>
+        </is>
+      </c>
+      <c r="K2" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H2" s="29" t="inlineStr">
+      <c r="L2" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4869,6 +4892,16 @@
         <is>
           <t>Blank 8
 Right Branching Condition</t>
+        </is>
+      </c>
+      <c r="K3" s="58" t="inlineStr">
+        <is>
+          <t>Overall WS3</t>
+        </is>
+      </c>
+      <c r="L3" s="58" t="inlineStr">
+        <is>
+          <t>Notes WS3</t>
         </is>
       </c>
     </row>
@@ -5702,6 +5735,7 @@
       <c r="G51" s="45" t="n"/>
       <c r="H51" s="46" t="n"/>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="48" t="inlineStr">
         <is>
@@ -5759,12 +5793,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A4:H4"/>
     <mergeCell ref="A53:H53"/>
-    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="A36:H36"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A35:L35"/>
+    <mergeCell ref="A4:L4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 F48 F49 F50 F51 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47 G48 G49 G50 G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose: Acquire, Deepen, Create, or ?" promptTitle="Select level" prompt="AI-CFT level" type="list">

</xml_diff>

<commit_message>
WS3: fix AI-CFT levels - Blank 1-6 Acquire, Blank 7-8 Deepen
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -4799,29 +4799,29 @@
           <t>Acquire</t>
         </is>
       </c>
-      <c r="F2" s="30" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>Acquire</t>
+        </is>
+      </c>
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>Acquire</t>
+        </is>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>Acquire</t>
+        </is>
+      </c>
+      <c r="I2" s="30" t="inlineStr">
         <is>
           <t>Deepen</t>
         </is>
       </c>
-      <c r="G2" s="28" t="inlineStr">
-        <is>
-          <t>Acquire</t>
-        </is>
-      </c>
-      <c r="H2" s="28" t="inlineStr">
-        <is>
-          <t>Acquire</t>
-        </is>
-      </c>
-      <c r="I2" s="28" t="inlineStr">
-        <is>
-          <t>Acquire</t>
-        </is>
-      </c>
-      <c r="J2" s="28" t="inlineStr">
-        <is>
-          <t>Acquire</t>
+      <c r="J2" s="30" t="inlineStr">
+        <is>
+          <t>Deepen</t>
         </is>
       </c>
       <c r="K2" s="29" t="inlineStr">
@@ -5735,7 +5735,6 @@
       <c r="G51" s="45" t="n"/>
       <c r="H51" s="46" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
WS3: expand all column widths
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -4760,10 +4760,17 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="36" min="1" max="1"/>
-    <col width="18" customWidth="1" style="36" min="2" max="2"/>
-    <col width="13" customWidth="1" style="36" min="3" max="6"/>
-    <col width="14" customWidth="1" style="36" min="7" max="7"/>
-    <col width="40" customWidth="1" style="36" min="8" max="8"/>
+    <col width="16" customWidth="1" style="36" min="2" max="2"/>
+    <col width="22" customWidth="1" style="36" min="3" max="6"/>
+    <col width="22" customWidth="1" style="36" min="4" max="4"/>
+    <col width="22" customWidth="1" style="36" min="5" max="5"/>
+    <col width="22" customWidth="1" style="36" min="6" max="6"/>
+    <col width="22" customWidth="1" style="36" min="7" max="7"/>
+    <col width="22" customWidth="1" style="36" min="8" max="8"/>
+    <col width="22" customWidth="1" style="36" min="9" max="9"/>
+    <col width="22" customWidth="1" style="36" min="10" max="10"/>
+    <col width="14" customWidth="1" style="36" min="11" max="11"/>
+    <col width="20" customWidth="1" style="36" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="36">
@@ -4835,7 +4842,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" s="36">
+    <row r="3" ht="50" customHeight="1" s="36">
       <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Cohort</t>

</xml_diff>

<commit_message>
WS3: apply full reference color scheme and column widths
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,8 +131,28 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00595959"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -182,6 +202,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF4FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -241,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -402,6 +452,60 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4761,986 +4865,1170 @@
   <cols>
     <col width="10" customWidth="1" style="36" min="1" max="1"/>
     <col width="16" customWidth="1" style="36" min="2" max="2"/>
-    <col width="22" customWidth="1" style="36" min="3" max="6"/>
-    <col width="22" customWidth="1" style="36" min="4" max="4"/>
-    <col width="22" customWidth="1" style="36" min="5" max="5"/>
-    <col width="22" customWidth="1" style="36" min="6" max="6"/>
-    <col width="22" customWidth="1" style="36" min="7" max="7"/>
-    <col width="22" customWidth="1" style="36" min="8" max="8"/>
-    <col width="22" customWidth="1" style="36" min="9" max="9"/>
-    <col width="22" customWidth="1" style="36" min="10" max="10"/>
+    <col width="20" customWidth="1" style="36" min="3" max="6"/>
+    <col width="20" customWidth="1" style="36" min="4" max="4"/>
+    <col width="20" customWidth="1" style="36" min="5" max="5"/>
+    <col width="20" customWidth="1" style="36" min="6" max="6"/>
+    <col width="20" customWidth="1" style="36" min="7" max="7"/>
+    <col width="20" customWidth="1" style="36" min="8" max="8"/>
+    <col width="20" customWidth="1" style="36" min="9" max="9"/>
+    <col width="20" customWidth="1" style="36" min="10" max="10"/>
     <col width="14" customWidth="1" style="36" min="11" max="11"/>
-    <col width="20" customWidth="1" style="36" min="12" max="12"/>
+    <col width="22" customWidth="1" style="36" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="36">
-      <c r="A1" s="47" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>AI-CFT Labeling — WS3 - Threshold Apply</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" s="36">
-      <c r="A2" s="27" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>Cohort</t>
         </is>
       </c>
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>Student</t>
         </is>
       </c>
-      <c r="C2" s="28" t="inlineStr">
+      <c r="C2" s="61" t="inlineStr">
         <is>
           <t>Acquire</t>
         </is>
       </c>
-      <c r="D2" s="28" t="inlineStr">
+      <c r="D2" s="61" t="inlineStr">
         <is>
           <t>Acquire</t>
         </is>
       </c>
-      <c r="E2" s="28" t="inlineStr">
+      <c r="E2" s="61" t="inlineStr">
         <is>
           <t>Acquire</t>
         </is>
       </c>
-      <c r="F2" s="28" t="inlineStr">
+      <c r="F2" s="61" t="inlineStr">
         <is>
           <t>Acquire</t>
         </is>
       </c>
-      <c r="G2" s="28" t="inlineStr">
+      <c r="G2" s="61" t="inlineStr">
         <is>
           <t>Acquire</t>
         </is>
       </c>
-      <c r="H2" s="28" t="inlineStr">
+      <c r="H2" s="61" t="inlineStr">
         <is>
           <t>Acquire</t>
         </is>
       </c>
-      <c r="I2" s="30" t="inlineStr">
+      <c r="I2" s="62" t="inlineStr">
         <is>
           <t>Deepen</t>
         </is>
       </c>
-      <c r="J2" s="30" t="inlineStr">
+      <c r="J2" s="62" t="inlineStr">
         <is>
           <t>Deepen</t>
         </is>
       </c>
-      <c r="K2" s="29" t="inlineStr">
+      <c r="K2" s="63" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L2" s="29" t="inlineStr">
+      <c r="L2" s="63" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="50" customHeight="1" s="36">
-      <c r="A3" s="15" t="inlineStr">
+    <row r="3" ht="48" customHeight="1" s="36">
+      <c r="A3" s="64" t="inlineStr">
         <is>
           <t>Cohort</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="64" t="inlineStr">
         <is>
           <t>Student Name</t>
         </is>
       </c>
-      <c r="C3" s="56" t="inlineStr">
+      <c r="C3" s="65" t="inlineStr">
         <is>
           <t>Blank 1
 Instance Classification (Popcorn)</t>
         </is>
       </c>
-      <c r="D3" s="56" t="inlineStr">
+      <c r="D3" s="65" t="inlineStr">
         <is>
           <t>Blank 2
 Rule Verification (Popcorn)</t>
         </is>
       </c>
-      <c r="E3" s="56" t="inlineStr">
+      <c r="E3" s="65" t="inlineStr">
         <is>
           <t>Blank 3
 Instance Classification (Apple)</t>
         </is>
       </c>
-      <c r="F3" s="56" t="inlineStr">
+      <c r="F3" s="65" t="inlineStr">
         <is>
           <t>Blank 4
 Rule Verification (Apple)</t>
         </is>
       </c>
-      <c r="G3" s="56" t="inlineStr">
+      <c r="G3" s="65" t="inlineStr">
         <is>
           <t>Blank 5
 Instance Classification (French Fries)</t>
         </is>
       </c>
-      <c r="H3" s="56" t="inlineStr">
+      <c r="H3" s="65" t="inlineStr">
         <is>
           <t>Blank 6
 Rule Verification (French Fries)</t>
         </is>
       </c>
-      <c r="I3" s="57" t="inlineStr">
+      <c r="I3" s="66" t="inlineStr">
         <is>
           <t>Blank 7
 Left Branching Condition</t>
         </is>
       </c>
-      <c r="J3" s="57" t="inlineStr">
+      <c r="J3" s="66" t="inlineStr">
         <is>
           <t>Blank 8
 Right Branching Condition</t>
         </is>
       </c>
-      <c r="K3" s="58" t="inlineStr">
+      <c r="K3" s="66" t="inlineStr">
         <is>
           <t>Overall WS3</t>
         </is>
       </c>
-      <c r="L3" s="58" t="inlineStr">
+      <c r="L3" s="66" t="inlineStr">
         <is>
           <t>Notes WS3</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1" s="36">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="4" ht="20" customHeight="1" s="36">
+      <c r="A4" s="67" t="inlineStr">
         <is>
           <t>▶  Cohort 2025</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" s="36">
-      <c r="A5" s="49" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B5" s="33" t="n"/>
-      <c r="C5" s="33" t="n"/>
-      <c r="D5" s="33" t="n"/>
-      <c r="E5" s="33" t="n"/>
-      <c r="F5" s="33" t="n"/>
-      <c r="G5" s="33" t="n"/>
-      <c r="H5" s="34" t="n"/>
+      <c r="A5" s="68" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="69" t="n"/>
+      <c r="C5" s="69" t="n"/>
+      <c r="D5" s="69" t="n"/>
+      <c r="E5" s="69" t="n"/>
+      <c r="F5" s="69" t="n"/>
+      <c r="G5" s="69" t="n"/>
+      <c r="H5" s="68" t="n"/>
+      <c r="I5" s="70" t="n"/>
+      <c r="J5" s="70" t="n"/>
+      <c r="K5" s="71" t="n"/>
+      <c r="L5" s="71" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="36">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="A6" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B6" s="72" t="inlineStr">
         <is>
           <t>Ally</t>
         </is>
       </c>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="45" t="n"/>
-      <c r="H6" s="46" t="n"/>
+      <c r="C6" s="73" t="n"/>
+      <c r="D6" s="73" t="n"/>
+      <c r="E6" s="73" t="n"/>
+      <c r="F6" s="73" t="n"/>
+      <c r="G6" s="73" t="n"/>
+      <c r="H6" s="73" t="n"/>
+      <c r="I6" s="72" t="n"/>
+      <c r="J6" s="72" t="n"/>
+      <c r="K6" s="71" t="n"/>
+      <c r="L6" s="71" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1" s="36">
-      <c r="A7" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B7" s="43" t="inlineStr">
+      <c r="A7" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B7" s="70" t="inlineStr">
         <is>
           <t>Bella</t>
         </is>
       </c>
-      <c r="C7" s="44" t="n"/>
-      <c r="D7" s="44" t="n"/>
-      <c r="E7" s="44" t="n"/>
-      <c r="F7" s="44" t="n"/>
-      <c r="G7" s="45" t="n"/>
-      <c r="H7" s="46" t="n"/>
+      <c r="C7" s="74" t="n"/>
+      <c r="D7" s="74" t="n"/>
+      <c r="E7" s="74" t="n"/>
+      <c r="F7" s="74" t="n"/>
+      <c r="G7" s="74" t="n"/>
+      <c r="H7" s="74" t="n"/>
+      <c r="I7" s="70" t="n"/>
+      <c r="J7" s="70" t="n"/>
+      <c r="K7" s="71" t="n"/>
+      <c r="L7" s="71" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="36">
-      <c r="A8" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="A8" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B8" s="72" t="inlineStr">
         <is>
           <t>Bob</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="45" t="n"/>
-      <c r="H8" s="46" t="n"/>
+      <c r="C8" s="73" t="n"/>
+      <c r="D8" s="73" t="n"/>
+      <c r="E8" s="73" t="n"/>
+      <c r="F8" s="73" t="n"/>
+      <c r="G8" s="73" t="n"/>
+      <c r="H8" s="73" t="n"/>
+      <c r="I8" s="72" t="n"/>
+      <c r="J8" s="72" t="n"/>
+      <c r="K8" s="71" t="n"/>
+      <c r="L8" s="71" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1" s="36">
-      <c r="A9" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B9" s="43" t="inlineStr">
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B9" s="70" t="inlineStr">
         <is>
           <t>Daisy</t>
         </is>
       </c>
-      <c r="C9" s="44" t="n"/>
-      <c r="D9" s="44" t="n"/>
-      <c r="E9" s="44" t="n"/>
-      <c r="F9" s="44" t="n"/>
-      <c r="G9" s="45" t="n"/>
-      <c r="H9" s="46" t="n"/>
+      <c r="C9" s="74" t="n"/>
+      <c r="D9" s="74" t="n"/>
+      <c r="E9" s="74" t="n"/>
+      <c r="F9" s="74" t="n"/>
+      <c r="G9" s="74" t="n"/>
+      <c r="H9" s="74" t="n"/>
+      <c r="I9" s="70" t="n"/>
+      <c r="J9" s="70" t="n"/>
+      <c r="K9" s="71" t="n"/>
+      <c r="L9" s="71" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1" s="36">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="A10" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B10" s="72" t="inlineStr">
         <is>
           <t>Daniella</t>
         </is>
       </c>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="24" t="n"/>
-      <c r="F10" s="24" t="n"/>
-      <c r="G10" s="45" t="n"/>
-      <c r="H10" s="46" t="n"/>
+      <c r="C10" s="73" t="n"/>
+      <c r="D10" s="73" t="n"/>
+      <c r="E10" s="73" t="n"/>
+      <c r="F10" s="73" t="n"/>
+      <c r="G10" s="73" t="n"/>
+      <c r="H10" s="73" t="n"/>
+      <c r="I10" s="72" t="n"/>
+      <c r="J10" s="72" t="n"/>
+      <c r="K10" s="71" t="n"/>
+      <c r="L10" s="71" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1" s="36">
-      <c r="A11" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B11" s="70" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
-      <c r="C11" s="44" t="n"/>
-      <c r="D11" s="44" t="n"/>
-      <c r="E11" s="44" t="n"/>
-      <c r="F11" s="44" t="n"/>
-      <c r="G11" s="45" t="n"/>
-      <c r="H11" s="46" t="n"/>
+      <c r="C11" s="74" t="n"/>
+      <c r="D11" s="74" t="n"/>
+      <c r="E11" s="74" t="n"/>
+      <c r="F11" s="74" t="n"/>
+      <c r="G11" s="74" t="n"/>
+      <c r="H11" s="74" t="n"/>
+      <c r="I11" s="70" t="n"/>
+      <c r="J11" s="70" t="n"/>
+      <c r="K11" s="71" t="n"/>
+      <c r="L11" s="71" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1" s="36">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="A12" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B12" s="72" t="inlineStr">
         <is>
           <t>Eliot</t>
         </is>
       </c>
-      <c r="C12" s="24" t="n"/>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="24" t="n"/>
-      <c r="F12" s="24" t="n"/>
-      <c r="G12" s="45" t="n"/>
-      <c r="H12" s="46" t="n"/>
+      <c r="C12" s="73" t="n"/>
+      <c r="D12" s="73" t="n"/>
+      <c r="E12" s="73" t="n"/>
+      <c r="F12" s="73" t="n"/>
+      <c r="G12" s="73" t="n"/>
+      <c r="H12" s="73" t="n"/>
+      <c r="I12" s="72" t="n"/>
+      <c r="J12" s="72" t="n"/>
+      <c r="K12" s="71" t="n"/>
+      <c r="L12" s="71" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1" s="36">
-      <c r="A13" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="A13" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="inlineStr">
         <is>
           <t>Henry</t>
         </is>
       </c>
-      <c r="C13" s="44" t="n"/>
-      <c r="D13" s="44" t="n"/>
-      <c r="E13" s="44" t="n"/>
-      <c r="F13" s="44" t="n"/>
-      <c r="G13" s="45" t="n"/>
-      <c r="H13" s="46" t="n"/>
+      <c r="C13" s="74" t="n"/>
+      <c r="D13" s="74" t="n"/>
+      <c r="E13" s="74" t="n"/>
+      <c r="F13" s="74" t="n"/>
+      <c r="G13" s="74" t="n"/>
+      <c r="H13" s="74" t="n"/>
+      <c r="I13" s="70" t="n"/>
+      <c r="J13" s="70" t="n"/>
+      <c r="K13" s="71" t="n"/>
+      <c r="L13" s="71" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1" s="36">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="A14" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B14" s="72" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="24" t="n"/>
-      <c r="G14" s="45" t="n"/>
-      <c r="H14" s="46" t="n"/>
+      <c r="C14" s="73" t="n"/>
+      <c r="D14" s="73" t="n"/>
+      <c r="E14" s="73" t="n"/>
+      <c r="F14" s="73" t="n"/>
+      <c r="G14" s="73" t="n"/>
+      <c r="H14" s="73" t="n"/>
+      <c r="I14" s="72" t="n"/>
+      <c r="J14" s="72" t="n"/>
+      <c r="K14" s="71" t="n"/>
+      <c r="L14" s="71" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1" s="36">
-      <c r="A15" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B15" s="43" t="inlineStr">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B15" s="70" t="inlineStr">
         <is>
           <t>Isabel</t>
         </is>
       </c>
-      <c r="C15" s="44" t="n"/>
-      <c r="D15" s="44" t="n"/>
-      <c r="E15" s="44" t="n"/>
-      <c r="F15" s="44" t="n"/>
-      <c r="G15" s="45" t="n"/>
-      <c r="H15" s="46" t="n"/>
+      <c r="C15" s="74" t="n"/>
+      <c r="D15" s="74" t="n"/>
+      <c r="E15" s="74" t="n"/>
+      <c r="F15" s="74" t="n"/>
+      <c r="G15" s="74" t="n"/>
+      <c r="H15" s="74" t="n"/>
+      <c r="I15" s="70" t="n"/>
+      <c r="J15" s="70" t="n"/>
+      <c r="K15" s="71" t="n"/>
+      <c r="L15" s="71" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1" s="36">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="A16" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B16" s="72" t="inlineStr">
         <is>
           <t>Karl</t>
         </is>
       </c>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="24" t="n"/>
-      <c r="G16" s="45" t="n"/>
-      <c r="H16" s="46" t="n"/>
+      <c r="C16" s="73" t="n"/>
+      <c r="D16" s="73" t="n"/>
+      <c r="E16" s="73" t="n"/>
+      <c r="F16" s="73" t="n"/>
+      <c r="G16" s="73" t="n"/>
+      <c r="H16" s="73" t="n"/>
+      <c r="I16" s="72" t="n"/>
+      <c r="J16" s="72" t="n"/>
+      <c r="K16" s="71" t="n"/>
+      <c r="L16" s="71" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1" s="36">
-      <c r="A17" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B17" s="43" t="inlineStr">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B17" s="70" t="inlineStr">
         <is>
           <t>Michael</t>
         </is>
       </c>
-      <c r="C17" s="44" t="n"/>
-      <c r="D17" s="44" t="n"/>
-      <c r="E17" s="44" t="n"/>
-      <c r="F17" s="44" t="n"/>
-      <c r="G17" s="45" t="n"/>
-      <c r="H17" s="46" t="n"/>
+      <c r="C17" s="74" t="n"/>
+      <c r="D17" s="74" t="n"/>
+      <c r="E17" s="74" t="n"/>
+      <c r="F17" s="74" t="n"/>
+      <c r="G17" s="74" t="n"/>
+      <c r="H17" s="74" t="n"/>
+      <c r="I17" s="70" t="n"/>
+      <c r="J17" s="70" t="n"/>
+      <c r="K17" s="71" t="n"/>
+      <c r="L17" s="71" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1" s="36">
-      <c r="A18" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="A18" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B18" s="72" t="inlineStr">
         <is>
           <t>Mike</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="24" t="n"/>
-      <c r="F18" s="24" t="n"/>
-      <c r="G18" s="45" t="n"/>
-      <c r="H18" s="46" t="n"/>
+      <c r="C18" s="73" t="n"/>
+      <c r="D18" s="73" t="n"/>
+      <c r="E18" s="73" t="n"/>
+      <c r="F18" s="73" t="n"/>
+      <c r="G18" s="73" t="n"/>
+      <c r="H18" s="73" t="n"/>
+      <c r="I18" s="72" t="n"/>
+      <c r="J18" s="72" t="n"/>
+      <c r="K18" s="71" t="n"/>
+      <c r="L18" s="71" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1" s="36">
-      <c r="A19" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B19" s="43" t="inlineStr">
+      <c r="A19" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B19" s="70" t="inlineStr">
         <is>
           <t>Nicolas</t>
         </is>
       </c>
-      <c r="C19" s="44" t="n"/>
-      <c r="D19" s="44" t="n"/>
-      <c r="E19" s="44" t="n"/>
-      <c r="F19" s="44" t="n"/>
-      <c r="G19" s="45" t="n"/>
-      <c r="H19" s="46" t="n"/>
+      <c r="C19" s="74" t="n"/>
+      <c r="D19" s="74" t="n"/>
+      <c r="E19" s="74" t="n"/>
+      <c r="F19" s="74" t="n"/>
+      <c r="G19" s="74" t="n"/>
+      <c r="H19" s="74" t="n"/>
+      <c r="I19" s="70" t="n"/>
+      <c r="J19" s="70" t="n"/>
+      <c r="K19" s="71" t="n"/>
+      <c r="L19" s="71" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1" s="36">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="A20" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B20" s="72" t="inlineStr">
         <is>
           <t>Zabby</t>
         </is>
       </c>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="45" t="n"/>
-      <c r="H20" s="46" t="n"/>
+      <c r="C20" s="73" t="n"/>
+      <c r="D20" s="73" t="n"/>
+      <c r="E20" s="73" t="n"/>
+      <c r="F20" s="73" t="n"/>
+      <c r="G20" s="73" t="n"/>
+      <c r="H20" s="73" t="n"/>
+      <c r="I20" s="72" t="n"/>
+      <c r="J20" s="72" t="n"/>
+      <c r="K20" s="71" t="n"/>
+      <c r="L20" s="71" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1" s="36">
-      <c r="A21" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B21" s="43" t="inlineStr">
+      <c r="A21" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B21" s="70" t="inlineStr">
         <is>
           <t>Adam</t>
         </is>
       </c>
-      <c r="C21" s="44" t="n"/>
-      <c r="D21" s="44" t="n"/>
-      <c r="E21" s="44" t="n"/>
-      <c r="F21" s="44" t="n"/>
-      <c r="G21" s="45" t="n"/>
-      <c r="H21" s="46" t="n"/>
+      <c r="C21" s="74" t="n"/>
+      <c r="D21" s="74" t="n"/>
+      <c r="E21" s="74" t="n"/>
+      <c r="F21" s="74" t="n"/>
+      <c r="G21" s="74" t="n"/>
+      <c r="H21" s="74" t="n"/>
+      <c r="I21" s="70" t="n"/>
+      <c r="J21" s="70" t="n"/>
+      <c r="K21" s="71" t="n"/>
+      <c r="L21" s="71" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1" s="36">
-      <c r="A22" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="A22" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B22" s="72" t="inlineStr">
         <is>
           <t>Eddy</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24" t="n"/>
-      <c r="F22" s="24" t="n"/>
-      <c r="G22" s="45" t="n"/>
-      <c r="H22" s="46" t="n"/>
+      <c r="C22" s="73" t="n"/>
+      <c r="D22" s="73" t="n"/>
+      <c r="E22" s="73" t="n"/>
+      <c r="F22" s="73" t="n"/>
+      <c r="G22" s="73" t="n"/>
+      <c r="H22" s="73" t="n"/>
+      <c r="I22" s="72" t="n"/>
+      <c r="J22" s="72" t="n"/>
+      <c r="K22" s="71" t="n"/>
+      <c r="L22" s="71" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="36">
-      <c r="A23" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B23" s="43" t="inlineStr">
+      <c r="A23" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B23" s="70" t="inlineStr">
         <is>
           <t>Aden</t>
         </is>
       </c>
-      <c r="C23" s="44" t="n"/>
-      <c r="D23" s="44" t="n"/>
-      <c r="E23" s="44" t="n"/>
-      <c r="F23" s="44" t="n"/>
-      <c r="G23" s="45" t="n"/>
-      <c r="H23" s="46" t="n"/>
+      <c r="C23" s="74" t="n"/>
+      <c r="D23" s="74" t="n"/>
+      <c r="E23" s="74" t="n"/>
+      <c r="F23" s="74" t="n"/>
+      <c r="G23" s="74" t="n"/>
+      <c r="H23" s="74" t="n"/>
+      <c r="I23" s="70" t="n"/>
+      <c r="J23" s="70" t="n"/>
+      <c r="K23" s="71" t="n"/>
+      <c r="L23" s="71" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1" s="36">
-      <c r="A24" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="A24" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B24" s="72" t="inlineStr">
         <is>
           <t>Barbara</t>
         </is>
       </c>
-      <c r="C24" s="24" t="n"/>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="24" t="n"/>
-      <c r="G24" s="45" t="n"/>
-      <c r="H24" s="46" t="n"/>
+      <c r="C24" s="73" t="n"/>
+      <c r="D24" s="73" t="n"/>
+      <c r="E24" s="73" t="n"/>
+      <c r="F24" s="73" t="n"/>
+      <c r="G24" s="73" t="n"/>
+      <c r="H24" s="73" t="n"/>
+      <c r="I24" s="72" t="n"/>
+      <c r="J24" s="72" t="n"/>
+      <c r="K24" s="71" t="n"/>
+      <c r="L24" s="71" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1" s="36">
-      <c r="A25" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B25" s="43" t="inlineStr">
+      <c r="A25" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B25" s="70" t="inlineStr">
         <is>
           <t>Boris</t>
         </is>
       </c>
-      <c r="C25" s="44" t="n"/>
-      <c r="D25" s="44" t="n"/>
-      <c r="E25" s="44" t="n"/>
-      <c r="F25" s="44" t="n"/>
-      <c r="G25" s="45" t="n"/>
-      <c r="H25" s="46" t="n"/>
+      <c r="C25" s="74" t="n"/>
+      <c r="D25" s="74" t="n"/>
+      <c r="E25" s="74" t="n"/>
+      <c r="F25" s="74" t="n"/>
+      <c r="G25" s="74" t="n"/>
+      <c r="H25" s="74" t="n"/>
+      <c r="I25" s="70" t="n"/>
+      <c r="J25" s="70" t="n"/>
+      <c r="K25" s="71" t="n"/>
+      <c r="L25" s="71" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="36">
-      <c r="A26" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B26" s="72" t="inlineStr">
         <is>
           <t>Calvin</t>
         </is>
       </c>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
-      <c r="G26" s="45" t="n"/>
-      <c r="H26" s="46" t="n"/>
+      <c r="C26" s="73" t="n"/>
+      <c r="D26" s="73" t="n"/>
+      <c r="E26" s="73" t="n"/>
+      <c r="F26" s="73" t="n"/>
+      <c r="G26" s="73" t="n"/>
+      <c r="H26" s="73" t="n"/>
+      <c r="I26" s="72" t="n"/>
+      <c r="J26" s="72" t="n"/>
+      <c r="K26" s="71" t="n"/>
+      <c r="L26" s="71" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1" s="36">
-      <c r="A27" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B27" s="43" t="inlineStr">
+      <c r="A27" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B27" s="70" t="inlineStr">
         <is>
           <t>Darby</t>
         </is>
       </c>
-      <c r="C27" s="44" t="n"/>
-      <c r="D27" s="44" t="n"/>
-      <c r="E27" s="44" t="n"/>
-      <c r="F27" s="44" t="n"/>
-      <c r="G27" s="45" t="n"/>
-      <c r="H27" s="46" t="n"/>
+      <c r="C27" s="74" t="n"/>
+      <c r="D27" s="74" t="n"/>
+      <c r="E27" s="74" t="n"/>
+      <c r="F27" s="74" t="n"/>
+      <c r="G27" s="74" t="n"/>
+      <c r="H27" s="74" t="n"/>
+      <c r="I27" s="70" t="n"/>
+      <c r="J27" s="70" t="n"/>
+      <c r="K27" s="71" t="n"/>
+      <c r="L27" s="71" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1" s="36">
-      <c r="A28" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B28" s="23" t="inlineStr">
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B28" s="72" t="inlineStr">
         <is>
           <t>Demi</t>
         </is>
       </c>
-      <c r="C28" s="24" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="24" t="n"/>
-      <c r="F28" s="24" t="n"/>
-      <c r="G28" s="45" t="n"/>
-      <c r="H28" s="46" t="n"/>
+      <c r="C28" s="73" t="n"/>
+      <c r="D28" s="73" t="n"/>
+      <c r="E28" s="73" t="n"/>
+      <c r="F28" s="73" t="n"/>
+      <c r="G28" s="73" t="n"/>
+      <c r="H28" s="73" t="n"/>
+      <c r="I28" s="72" t="n"/>
+      <c r="J28" s="72" t="n"/>
+      <c r="K28" s="71" t="n"/>
+      <c r="L28" s="71" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1" s="36">
-      <c r="A29" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B29" s="43" t="inlineStr">
+      <c r="A29" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B29" s="70" t="inlineStr">
         <is>
           <t>Daryl</t>
         </is>
       </c>
-      <c r="C29" s="44" t="n"/>
-      <c r="D29" s="44" t="n"/>
-      <c r="E29" s="44" t="n"/>
-      <c r="F29" s="44" t="n"/>
-      <c r="G29" s="45" t="n"/>
-      <c r="H29" s="46" t="n"/>
+      <c r="C29" s="74" t="n"/>
+      <c r="D29" s="74" t="n"/>
+      <c r="E29" s="74" t="n"/>
+      <c r="F29" s="74" t="n"/>
+      <c r="G29" s="74" t="n"/>
+      <c r="H29" s="74" t="n"/>
+      <c r="I29" s="70" t="n"/>
+      <c r="J29" s="70" t="n"/>
+      <c r="K29" s="71" t="n"/>
+      <c r="L29" s="71" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1" s="36">
-      <c r="A30" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B30" s="23" t="inlineStr">
+      <c r="A30" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B30" s="72" t="inlineStr">
         <is>
           <t>Edgar</t>
         </is>
       </c>
-      <c r="C30" s="24" t="n"/>
-      <c r="D30" s="24" t="n"/>
-      <c r="E30" s="24" t="n"/>
-      <c r="F30" s="24" t="n"/>
-      <c r="G30" s="45" t="n"/>
-      <c r="H30" s="46" t="n"/>
+      <c r="C30" s="73" t="n"/>
+      <c r="D30" s="73" t="n"/>
+      <c r="E30" s="73" t="n"/>
+      <c r="F30" s="73" t="n"/>
+      <c r="G30" s="73" t="n"/>
+      <c r="H30" s="73" t="n"/>
+      <c r="I30" s="72" t="n"/>
+      <c r="J30" s="72" t="n"/>
+      <c r="K30" s="71" t="n"/>
+      <c r="L30" s="71" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1" s="36">
-      <c r="A31" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B31" s="43" t="inlineStr">
+      <c r="A31" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B31" s="70" t="inlineStr">
         <is>
           <t>Frank</t>
         </is>
       </c>
-      <c r="C31" s="44" t="n"/>
-      <c r="D31" s="44" t="n"/>
-      <c r="E31" s="44" t="n"/>
-      <c r="F31" s="44" t="n"/>
-      <c r="G31" s="45" t="n"/>
-      <c r="H31" s="46" t="n"/>
+      <c r="C31" s="74" t="n"/>
+      <c r="D31" s="74" t="n"/>
+      <c r="E31" s="74" t="n"/>
+      <c r="F31" s="74" t="n"/>
+      <c r="G31" s="74" t="n"/>
+      <c r="H31" s="74" t="n"/>
+      <c r="I31" s="70" t="n"/>
+      <c r="J31" s="70" t="n"/>
+      <c r="K31" s="71" t="n"/>
+      <c r="L31" s="71" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1" s="36">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B32" s="23" t="inlineStr">
+      <c r="A32" s="72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B32" s="72" t="inlineStr">
         <is>
           <t>Felicity</t>
         </is>
       </c>
-      <c r="C32" s="24" t="n"/>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
-      <c r="G32" s="45" t="n"/>
-      <c r="H32" s="46" t="n"/>
+      <c r="C32" s="73" t="n"/>
+      <c r="D32" s="73" t="n"/>
+      <c r="E32" s="73" t="n"/>
+      <c r="F32" s="73" t="n"/>
+      <c r="G32" s="73" t="n"/>
+      <c r="H32" s="73" t="n"/>
+      <c r="I32" s="72" t="n"/>
+      <c r="J32" s="72" t="n"/>
+      <c r="K32" s="71" t="n"/>
+      <c r="L32" s="71" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1" s="36">
-      <c r="A33" s="42" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B33" s="43" t="inlineStr">
+      <c r="A33" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B33" s="70" t="inlineStr">
         <is>
           <t>Kim</t>
         </is>
       </c>
-      <c r="C33" s="44" t="n"/>
-      <c r="D33" s="44" t="n"/>
-      <c r="E33" s="44" t="n"/>
-      <c r="F33" s="44" t="n"/>
-      <c r="G33" s="45" t="n"/>
-      <c r="H33" s="46" t="n"/>
+      <c r="C33" s="74" t="n"/>
+      <c r="D33" s="74" t="n"/>
+      <c r="E33" s="74" t="n"/>
+      <c r="F33" s="74" t="n"/>
+      <c r="G33" s="74" t="n"/>
+      <c r="H33" s="74" t="n"/>
+      <c r="I33" s="70" t="n"/>
+      <c r="J33" s="70" t="n"/>
+      <c r="K33" s="71" t="n"/>
+      <c r="L33" s="71" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1" s="36">
-      <c r="A34" s="32" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B34" s="33" t="n"/>
-      <c r="C34" s="33" t="n"/>
-      <c r="D34" s="33" t="n"/>
-      <c r="E34" s="33" t="n"/>
-      <c r="F34" s="33" t="n"/>
-      <c r="G34" s="33" t="n"/>
-      <c r="H34" s="34" t="n"/>
-    </row>
-    <row r="35" ht="18" customHeight="1" s="36">
-      <c r="A35" s="41" t="inlineStr">
+      <c r="A34" s="75" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B34" s="76" t="n"/>
+      <c r="C34" s="76" t="n"/>
+      <c r="D34" s="76" t="n"/>
+      <c r="E34" s="76" t="n"/>
+      <c r="F34" s="76" t="n"/>
+      <c r="G34" s="76" t="n"/>
+      <c r="H34" s="75" t="n"/>
+      <c r="I34" s="72" t="n"/>
+      <c r="J34" s="72" t="n"/>
+      <c r="K34" s="71" t="n"/>
+      <c r="L34" s="71" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" s="36">
+      <c r="A35" s="67" t="inlineStr">
         <is>
           <t>▶  Cohort 2026</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="36">
-      <c r="A36" s="49" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B36" s="33" t="n"/>
-      <c r="C36" s="33" t="n"/>
-      <c r="D36" s="33" t="n"/>
-      <c r="E36" s="33" t="n"/>
-      <c r="F36" s="33" t="n"/>
-      <c r="G36" s="33" t="n"/>
-      <c r="H36" s="34" t="n"/>
+      <c r="A36" s="68" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B36" s="69" t="n"/>
+      <c r="C36" s="69" t="n"/>
+      <c r="D36" s="69" t="n"/>
+      <c r="E36" s="69" t="n"/>
+      <c r="F36" s="69" t="n"/>
+      <c r="G36" s="69" t="n"/>
+      <c r="H36" s="68" t="n"/>
+      <c r="I36" s="70" t="n"/>
+      <c r="J36" s="70" t="n"/>
+      <c r="K36" s="71" t="n"/>
+      <c r="L36" s="71" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="36">
-      <c r="A37" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B37" s="23" t="inlineStr">
+      <c r="A37" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B37" s="72" t="inlineStr">
         <is>
           <t>Marco</t>
         </is>
       </c>
-      <c r="C37" s="24" t="n"/>
-      <c r="D37" s="24" t="n"/>
-      <c r="E37" s="24" t="n"/>
-      <c r="F37" s="24" t="n"/>
-      <c r="G37" s="45" t="n"/>
-      <c r="H37" s="46" t="n"/>
+      <c r="C37" s="73" t="n"/>
+      <c r="D37" s="73" t="n"/>
+      <c r="E37" s="73" t="n"/>
+      <c r="F37" s="73" t="n"/>
+      <c r="G37" s="73" t="n"/>
+      <c r="H37" s="73" t="n"/>
+      <c r="I37" s="72" t="n"/>
+      <c r="J37" s="72" t="n"/>
+      <c r="K37" s="71" t="n"/>
+      <c r="L37" s="71" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1" s="36">
-      <c r="A38" s="42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B38" s="43" t="inlineStr">
+      <c r="A38" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B38" s="70" t="inlineStr">
         <is>
           <t>Iris</t>
         </is>
       </c>
-      <c r="C38" s="44" t="n"/>
-      <c r="D38" s="44" t="n"/>
-      <c r="E38" s="44" t="n"/>
-      <c r="F38" s="44" t="n"/>
-      <c r="G38" s="45" t="n"/>
-      <c r="H38" s="46" t="n"/>
+      <c r="C38" s="74" t="n"/>
+      <c r="D38" s="74" t="n"/>
+      <c r="E38" s="74" t="n"/>
+      <c r="F38" s="74" t="n"/>
+      <c r="G38" s="74" t="n"/>
+      <c r="H38" s="74" t="n"/>
+      <c r="I38" s="70" t="n"/>
+      <c r="J38" s="70" t="n"/>
+      <c r="K38" s="71" t="n"/>
+      <c r="L38" s="71" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1" s="36">
-      <c r="A39" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B39" s="23" t="inlineStr">
+      <c r="A39" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B39" s="72" t="inlineStr">
         <is>
           <t>Marcus</t>
         </is>
       </c>
-      <c r="C39" s="24" t="n"/>
-      <c r="D39" s="24" t="n"/>
-      <c r="E39" s="24" t="n"/>
-      <c r="F39" s="24" t="n"/>
-      <c r="G39" s="45" t="n"/>
-      <c r="H39" s="46" t="n"/>
+      <c r="C39" s="73" t="n"/>
+      <c r="D39" s="73" t="n"/>
+      <c r="E39" s="73" t="n"/>
+      <c r="F39" s="73" t="n"/>
+      <c r="G39" s="73" t="n"/>
+      <c r="H39" s="73" t="n"/>
+      <c r="I39" s="72" t="n"/>
+      <c r="J39" s="72" t="n"/>
+      <c r="K39" s="71" t="n"/>
+      <c r="L39" s="71" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="36">
-      <c r="A40" s="42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B40" s="43" t="inlineStr">
+      <c r="A40" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B40" s="70" t="inlineStr">
         <is>
           <t>Isabel</t>
         </is>
       </c>
-      <c r="C40" s="44" t="n"/>
-      <c r="D40" s="44" t="n"/>
-      <c r="E40" s="44" t="n"/>
-      <c r="F40" s="44" t="n"/>
-      <c r="G40" s="45" t="n"/>
-      <c r="H40" s="46" t="n"/>
+      <c r="C40" s="74" t="n"/>
+      <c r="D40" s="74" t="n"/>
+      <c r="E40" s="74" t="n"/>
+      <c r="F40" s="74" t="n"/>
+      <c r="G40" s="74" t="n"/>
+      <c r="H40" s="74" t="n"/>
+      <c r="I40" s="70" t="n"/>
+      <c r="J40" s="70" t="n"/>
+      <c r="K40" s="71" t="n"/>
+      <c r="L40" s="71" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1" s="36">
-      <c r="A41" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B41" s="23" t="inlineStr">
+      <c r="A41" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B41" s="72" t="inlineStr">
         <is>
           <t>Amy</t>
         </is>
       </c>
-      <c r="C41" s="24" t="n"/>
-      <c r="D41" s="24" t="n"/>
-      <c r="E41" s="24" t="n"/>
-      <c r="F41" s="24" t="n"/>
-      <c r="G41" s="45" t="n"/>
-      <c r="H41" s="46" t="n"/>
+      <c r="C41" s="73" t="n"/>
+      <c r="D41" s="73" t="n"/>
+      <c r="E41" s="73" t="n"/>
+      <c r="F41" s="73" t="n"/>
+      <c r="G41" s="73" t="n"/>
+      <c r="H41" s="73" t="n"/>
+      <c r="I41" s="72" t="n"/>
+      <c r="J41" s="72" t="n"/>
+      <c r="K41" s="71" t="n"/>
+      <c r="L41" s="71" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1" s="36">
-      <c r="A42" s="42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B42" s="43" t="inlineStr">
+      <c r="A42" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B42" s="70" t="inlineStr">
         <is>
           <t>Serena</t>
         </is>
       </c>
-      <c r="C42" s="44" t="n"/>
-      <c r="D42" s="44" t="n"/>
-      <c r="E42" s="44" t="n"/>
-      <c r="F42" s="44" t="n"/>
-      <c r="G42" s="45" t="n"/>
-      <c r="H42" s="46" t="n"/>
+      <c r="C42" s="74" t="n"/>
+      <c r="D42" s="74" t="n"/>
+      <c r="E42" s="74" t="n"/>
+      <c r="F42" s="74" t="n"/>
+      <c r="G42" s="74" t="n"/>
+      <c r="H42" s="74" t="n"/>
+      <c r="I42" s="70" t="n"/>
+      <c r="J42" s="70" t="n"/>
+      <c r="K42" s="71" t="n"/>
+      <c r="L42" s="71" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1" s="36">
-      <c r="A43" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B43" s="23" t="inlineStr">
+      <c r="A43" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B43" s="72" t="inlineStr">
         <is>
           <t>Irma</t>
         </is>
       </c>
-      <c r="C43" s="24" t="n"/>
-      <c r="D43" s="24" t="n"/>
-      <c r="E43" s="24" t="n"/>
-      <c r="F43" s="24" t="n"/>
-      <c r="G43" s="45" t="n"/>
-      <c r="H43" s="46" t="n"/>
+      <c r="C43" s="73" t="n"/>
+      <c r="D43" s="73" t="n"/>
+      <c r="E43" s="73" t="n"/>
+      <c r="F43" s="73" t="n"/>
+      <c r="G43" s="73" t="n"/>
+      <c r="H43" s="73" t="n"/>
+      <c r="I43" s="72" t="n"/>
+      <c r="J43" s="72" t="n"/>
+      <c r="K43" s="71" t="n"/>
+      <c r="L43" s="71" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1" s="36">
-      <c r="A44" s="42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B44" s="43" t="inlineStr">
+      <c r="A44" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B44" s="70" t="inlineStr">
         <is>
           <t>Kate</t>
         </is>
       </c>
-      <c r="C44" s="44" t="n"/>
-      <c r="D44" s="44" t="n"/>
-      <c r="E44" s="44" t="n"/>
-      <c r="F44" s="44" t="n"/>
-      <c r="G44" s="45" t="n"/>
-      <c r="H44" s="46" t="n"/>
+      <c r="C44" s="74" t="n"/>
+      <c r="D44" s="74" t="n"/>
+      <c r="E44" s="74" t="n"/>
+      <c r="F44" s="74" t="n"/>
+      <c r="G44" s="74" t="n"/>
+      <c r="H44" s="74" t="n"/>
+      <c r="I44" s="70" t="n"/>
+      <c r="J44" s="70" t="n"/>
+      <c r="K44" s="71" t="n"/>
+      <c r="L44" s="71" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1" s="36">
-      <c r="A45" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B45" s="23" t="inlineStr">
+      <c r="A45" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B45" s="72" t="inlineStr">
         <is>
           <t>Bruno</t>
         </is>
       </c>
-      <c r="C45" s="24" t="n"/>
-      <c r="D45" s="24" t="n"/>
-      <c r="E45" s="24" t="n"/>
-      <c r="F45" s="24" t="n"/>
-      <c r="G45" s="45" t="n"/>
-      <c r="H45" s="46" t="n"/>
+      <c r="C45" s="73" t="n"/>
+      <c r="D45" s="73" t="n"/>
+      <c r="E45" s="73" t="n"/>
+      <c r="F45" s="73" t="n"/>
+      <c r="G45" s="73" t="n"/>
+      <c r="H45" s="73" t="n"/>
+      <c r="I45" s="72" t="n"/>
+      <c r="J45" s="72" t="n"/>
+      <c r="K45" s="71" t="n"/>
+      <c r="L45" s="71" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1" s="36">
-      <c r="A46" s="42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B46" s="43" t="inlineStr">
+      <c r="A46" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B46" s="70" t="inlineStr">
         <is>
           <t>Zara</t>
         </is>
       </c>
-      <c r="C46" s="44" t="n"/>
-      <c r="D46" s="44" t="n"/>
-      <c r="E46" s="44" t="n"/>
-      <c r="F46" s="44" t="n"/>
-      <c r="G46" s="45" t="n"/>
-      <c r="H46" s="46" t="n"/>
+      <c r="C46" s="74" t="n"/>
+      <c r="D46" s="74" t="n"/>
+      <c r="E46" s="74" t="n"/>
+      <c r="F46" s="74" t="n"/>
+      <c r="G46" s="74" t="n"/>
+      <c r="H46" s="74" t="n"/>
+      <c r="I46" s="70" t="n"/>
+      <c r="J46" s="70" t="n"/>
+      <c r="K46" s="71" t="n"/>
+      <c r="L46" s="71" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="36">
-      <c r="A47" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B47" s="23" t="inlineStr">
+      <c r="A47" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B47" s="72" t="inlineStr">
         <is>
           <t>Shana</t>
         </is>
       </c>
-      <c r="C47" s="24" t="n"/>
-      <c r="D47" s="24" t="n"/>
-      <c r="E47" s="24" t="n"/>
-      <c r="F47" s="24" t="n"/>
-      <c r="G47" s="45" t="n"/>
-      <c r="H47" s="46" t="n"/>
+      <c r="C47" s="73" t="n"/>
+      <c r="D47" s="73" t="n"/>
+      <c r="E47" s="73" t="n"/>
+      <c r="F47" s="73" t="n"/>
+      <c r="G47" s="73" t="n"/>
+      <c r="H47" s="73" t="n"/>
+      <c r="I47" s="72" t="n"/>
+      <c r="J47" s="72" t="n"/>
+      <c r="K47" s="71" t="n"/>
+      <c r="L47" s="71" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1" s="36">
-      <c r="A48" s="42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B48" s="43" t="inlineStr">
+      <c r="A48" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B48" s="70" t="inlineStr">
         <is>
           <t>Melinda</t>
         </is>
       </c>
-      <c r="C48" s="44" t="n"/>
-      <c r="D48" s="44" t="n"/>
-      <c r="E48" s="44" t="n"/>
-      <c r="F48" s="44" t="n"/>
-      <c r="G48" s="45" t="n"/>
-      <c r="H48" s="46" t="n"/>
+      <c r="C48" s="74" t="n"/>
+      <c r="D48" s="74" t="n"/>
+      <c r="E48" s="74" t="n"/>
+      <c r="F48" s="74" t="n"/>
+      <c r="G48" s="74" t="n"/>
+      <c r="H48" s="74" t="n"/>
+      <c r="I48" s="70" t="n"/>
+      <c r="J48" s="70" t="n"/>
+      <c r="K48" s="71" t="n"/>
+      <c r="L48" s="71" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1" s="36">
-      <c r="A49" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B49" s="23" t="inlineStr">
+      <c r="A49" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B49" s="72" t="inlineStr">
         <is>
           <t>Helena</t>
         </is>
       </c>
-      <c r="C49" s="24" t="n"/>
-      <c r="D49" s="24" t="n"/>
-      <c r="E49" s="24" t="n"/>
-      <c r="F49" s="24" t="n"/>
-      <c r="G49" s="45" t="n"/>
-      <c r="H49" s="46" t="n"/>
+      <c r="C49" s="73" t="n"/>
+      <c r="D49" s="73" t="n"/>
+      <c r="E49" s="73" t="n"/>
+      <c r="F49" s="73" t="n"/>
+      <c r="G49" s="73" t="n"/>
+      <c r="H49" s="73" t="n"/>
+      <c r="I49" s="72" t="n"/>
+      <c r="J49" s="72" t="n"/>
+      <c r="K49" s="71" t="n"/>
+      <c r="L49" s="71" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="36">
-      <c r="A50" s="42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B50" s="43" t="inlineStr">
+      <c r="A50" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B50" s="70" t="inlineStr">
         <is>
           <t>Nadia</t>
         </is>
       </c>
-      <c r="C50" s="44" t="n"/>
-      <c r="D50" s="44" t="n"/>
-      <c r="E50" s="44" t="n"/>
-      <c r="F50" s="44" t="n"/>
-      <c r="G50" s="45" t="n"/>
-      <c r="H50" s="46" t="n"/>
+      <c r="C50" s="74" t="n"/>
+      <c r="D50" s="74" t="n"/>
+      <c r="E50" s="74" t="n"/>
+      <c r="F50" s="74" t="n"/>
+      <c r="G50" s="74" t="n"/>
+      <c r="H50" s="74" t="n"/>
+      <c r="I50" s="70" t="n"/>
+      <c r="J50" s="70" t="n"/>
+      <c r="K50" s="71" t="n"/>
+      <c r="L50" s="71" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1" s="36">
-      <c r="A51" s="22" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B51" s="23" t="inlineStr">
+      <c r="A51" s="72" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B51" s="72" t="inlineStr">
         <is>
           <t>Ulysses</t>
         </is>
       </c>
-      <c r="C51" s="24" t="n"/>
-      <c r="D51" s="24" t="n"/>
-      <c r="E51" s="24" t="n"/>
-      <c r="F51" s="24" t="n"/>
-      <c r="G51" s="45" t="n"/>
-      <c r="H51" s="46" t="n"/>
+      <c r="C51" s="73" t="n"/>
+      <c r="D51" s="73" t="n"/>
+      <c r="E51" s="73" t="n"/>
+      <c r="F51" s="73" t="n"/>
+      <c r="G51" s="73" t="n"/>
+      <c r="H51" s="73" t="n"/>
+      <c r="I51" s="72" t="n"/>
+      <c r="J51" s="72" t="n"/>
+      <c r="K51" s="71" t="n"/>
+      <c r="L51" s="71" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="48" t="inlineStr">

</xml_diff>

<commit_message>
WS3: uniform alternating colors for all cols, center all text
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -152,7 +152,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -234,6 +234,11 @@
         <fgColor rgb="00EAF4FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -291,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -505,6 +510,33 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4947,70 +4979,70 @@
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" s="36">
-      <c r="A3" s="64" t="inlineStr">
+      <c r="A3" s="77" t="inlineStr">
         <is>
           <t>Cohort</t>
         </is>
       </c>
-      <c r="B3" s="64" t="inlineStr">
+      <c r="B3" s="77" t="inlineStr">
         <is>
           <t>Student Name</t>
         </is>
       </c>
-      <c r="C3" s="65" t="inlineStr">
+      <c r="C3" s="78" t="inlineStr">
         <is>
           <t>Blank 1
 Instance Classification (Popcorn)</t>
         </is>
       </c>
-      <c r="D3" s="65" t="inlineStr">
+      <c r="D3" s="78" t="inlineStr">
         <is>
           <t>Blank 2
 Rule Verification (Popcorn)</t>
         </is>
       </c>
-      <c r="E3" s="65" t="inlineStr">
+      <c r="E3" s="78" t="inlineStr">
         <is>
           <t>Blank 3
 Instance Classification (Apple)</t>
         </is>
       </c>
-      <c r="F3" s="65" t="inlineStr">
+      <c r="F3" s="78" t="inlineStr">
         <is>
           <t>Blank 4
 Rule Verification (Apple)</t>
         </is>
       </c>
-      <c r="G3" s="65" t="inlineStr">
+      <c r="G3" s="78" t="inlineStr">
         <is>
           <t>Blank 5
 Instance Classification (French Fries)</t>
         </is>
       </c>
-      <c r="H3" s="65" t="inlineStr">
+      <c r="H3" s="78" t="inlineStr">
         <is>
           <t>Blank 6
 Rule Verification (French Fries)</t>
         </is>
       </c>
-      <c r="I3" s="66" t="inlineStr">
+      <c r="I3" s="79" t="inlineStr">
         <is>
           <t>Blank 7
 Left Branching Condition</t>
         </is>
       </c>
-      <c r="J3" s="66" t="inlineStr">
+      <c r="J3" s="79" t="inlineStr">
         <is>
           <t>Blank 8
 Right Branching Condition</t>
         </is>
       </c>
-      <c r="K3" s="66" t="inlineStr">
+      <c r="K3" s="79" t="inlineStr">
         <is>
           <t>Overall WS3</t>
         </is>
       </c>
-      <c r="L3" s="66" t="inlineStr">
+      <c r="L3" s="79" t="inlineStr">
         <is>
           <t>Notes WS3</t>
         </is>
@@ -5029,39 +5061,39 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="69" t="n"/>
-      <c r="C5" s="69" t="n"/>
-      <c r="D5" s="69" t="n"/>
-      <c r="E5" s="69" t="n"/>
-      <c r="F5" s="69" t="n"/>
-      <c r="G5" s="69" t="n"/>
-      <c r="H5" s="68" t="n"/>
+      <c r="B5" s="80" t="n"/>
+      <c r="C5" s="80" t="n"/>
+      <c r="D5" s="80" t="n"/>
+      <c r="E5" s="80" t="n"/>
+      <c r="F5" s="80" t="n"/>
+      <c r="G5" s="80" t="n"/>
+      <c r="H5" s="81" t="n"/>
       <c r="I5" s="70" t="n"/>
       <c r="J5" s="70" t="n"/>
-      <c r="K5" s="71" t="n"/>
-      <c r="L5" s="71" t="n"/>
+      <c r="K5" s="70" t="n"/>
+      <c r="L5" s="70" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="36">
-      <c r="A6" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B6" s="72" t="inlineStr">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B6" s="82" t="inlineStr">
         <is>
           <t>Ally</t>
         </is>
       </c>
-      <c r="C6" s="73" t="n"/>
-      <c r="D6" s="73" t="n"/>
-      <c r="E6" s="73" t="n"/>
-      <c r="F6" s="73" t="n"/>
-      <c r="G6" s="73" t="n"/>
-      <c r="H6" s="73" t="n"/>
-      <c r="I6" s="72" t="n"/>
-      <c r="J6" s="72" t="n"/>
-      <c r="K6" s="71" t="n"/>
-      <c r="L6" s="71" t="n"/>
+      <c r="C6" s="83" t="n"/>
+      <c r="D6" s="83" t="n"/>
+      <c r="E6" s="83" t="n"/>
+      <c r="F6" s="83" t="n"/>
+      <c r="G6" s="83" t="n"/>
+      <c r="H6" s="83" t="n"/>
+      <c r="I6" s="82" t="n"/>
+      <c r="J6" s="82" t="n"/>
+      <c r="K6" s="82" t="n"/>
+      <c r="L6" s="82" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1" s="36">
       <c r="A7" s="70" t="inlineStr">
@@ -5082,30 +5114,30 @@
       <c r="H7" s="74" t="n"/>
       <c r="I7" s="70" t="n"/>
       <c r="J7" s="70" t="n"/>
-      <c r="K7" s="71" t="n"/>
-      <c r="L7" s="71" t="n"/>
+      <c r="K7" s="70" t="n"/>
+      <c r="L7" s="70" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="36">
-      <c r="A8" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B8" s="72" t="inlineStr">
+      <c r="A8" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B8" s="82" t="inlineStr">
         <is>
           <t>Bob</t>
         </is>
       </c>
-      <c r="C8" s="73" t="n"/>
-      <c r="D8" s="73" t="n"/>
-      <c r="E8" s="73" t="n"/>
-      <c r="F8" s="73" t="n"/>
-      <c r="G8" s="73" t="n"/>
-      <c r="H8" s="73" t="n"/>
-      <c r="I8" s="72" t="n"/>
-      <c r="J8" s="72" t="n"/>
-      <c r="K8" s="71" t="n"/>
-      <c r="L8" s="71" t="n"/>
+      <c r="C8" s="83" t="n"/>
+      <c r="D8" s="83" t="n"/>
+      <c r="E8" s="83" t="n"/>
+      <c r="F8" s="83" t="n"/>
+      <c r="G8" s="83" t="n"/>
+      <c r="H8" s="83" t="n"/>
+      <c r="I8" s="82" t="n"/>
+      <c r="J8" s="82" t="n"/>
+      <c r="K8" s="82" t="n"/>
+      <c r="L8" s="82" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1" s="36">
       <c r="A9" s="70" t="inlineStr">
@@ -5126,30 +5158,30 @@
       <c r="H9" s="74" t="n"/>
       <c r="I9" s="70" t="n"/>
       <c r="J9" s="70" t="n"/>
-      <c r="K9" s="71" t="n"/>
-      <c r="L9" s="71" t="n"/>
+      <c r="K9" s="70" t="n"/>
+      <c r="L9" s="70" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1" s="36">
-      <c r="A10" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B10" s="72" t="inlineStr">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B10" s="82" t="inlineStr">
         <is>
           <t>Daniella</t>
         </is>
       </c>
-      <c r="C10" s="73" t="n"/>
-      <c r="D10" s="73" t="n"/>
-      <c r="E10" s="73" t="n"/>
-      <c r="F10" s="73" t="n"/>
-      <c r="G10" s="73" t="n"/>
-      <c r="H10" s="73" t="n"/>
-      <c r="I10" s="72" t="n"/>
-      <c r="J10" s="72" t="n"/>
-      <c r="K10" s="71" t="n"/>
-      <c r="L10" s="71" t="n"/>
+      <c r="C10" s="83" t="n"/>
+      <c r="D10" s="83" t="n"/>
+      <c r="E10" s="83" t="n"/>
+      <c r="F10" s="83" t="n"/>
+      <c r="G10" s="83" t="n"/>
+      <c r="H10" s="83" t="n"/>
+      <c r="I10" s="82" t="n"/>
+      <c r="J10" s="82" t="n"/>
+      <c r="K10" s="82" t="n"/>
+      <c r="L10" s="82" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1" s="36">
       <c r="A11" s="70" t="inlineStr">
@@ -5170,30 +5202,30 @@
       <c r="H11" s="74" t="n"/>
       <c r="I11" s="70" t="n"/>
       <c r="J11" s="70" t="n"/>
-      <c r="K11" s="71" t="n"/>
-      <c r="L11" s="71" t="n"/>
+      <c r="K11" s="70" t="n"/>
+      <c r="L11" s="70" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1" s="36">
-      <c r="A12" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B12" s="72" t="inlineStr">
+      <c r="A12" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B12" s="82" t="inlineStr">
         <is>
           <t>Eliot</t>
         </is>
       </c>
-      <c r="C12" s="73" t="n"/>
-      <c r="D12" s="73" t="n"/>
-      <c r="E12" s="73" t="n"/>
-      <c r="F12" s="73" t="n"/>
-      <c r="G12" s="73" t="n"/>
-      <c r="H12" s="73" t="n"/>
-      <c r="I12" s="72" t="n"/>
-      <c r="J12" s="72" t="n"/>
-      <c r="K12" s="71" t="n"/>
-      <c r="L12" s="71" t="n"/>
+      <c r="C12" s="83" t="n"/>
+      <c r="D12" s="83" t="n"/>
+      <c r="E12" s="83" t="n"/>
+      <c r="F12" s="83" t="n"/>
+      <c r="G12" s="83" t="n"/>
+      <c r="H12" s="83" t="n"/>
+      <c r="I12" s="82" t="n"/>
+      <c r="J12" s="82" t="n"/>
+      <c r="K12" s="82" t="n"/>
+      <c r="L12" s="82" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1" s="36">
       <c r="A13" s="70" t="inlineStr">
@@ -5214,30 +5246,30 @@
       <c r="H13" s="74" t="n"/>
       <c r="I13" s="70" t="n"/>
       <c r="J13" s="70" t="n"/>
-      <c r="K13" s="71" t="n"/>
-      <c r="L13" s="71" t="n"/>
+      <c r="K13" s="70" t="n"/>
+      <c r="L13" s="70" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1" s="36">
-      <c r="A14" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B14" s="72" t="inlineStr">
+      <c r="A14" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B14" s="82" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="C14" s="73" t="n"/>
-      <c r="D14" s="73" t="n"/>
-      <c r="E14" s="73" t="n"/>
-      <c r="F14" s="73" t="n"/>
-      <c r="G14" s="73" t="n"/>
-      <c r="H14" s="73" t="n"/>
-      <c r="I14" s="72" t="n"/>
-      <c r="J14" s="72" t="n"/>
-      <c r="K14" s="71" t="n"/>
-      <c r="L14" s="71" t="n"/>
+      <c r="C14" s="83" t="n"/>
+      <c r="D14" s="83" t="n"/>
+      <c r="E14" s="83" t="n"/>
+      <c r="F14" s="83" t="n"/>
+      <c r="G14" s="83" t="n"/>
+      <c r="H14" s="83" t="n"/>
+      <c r="I14" s="82" t="n"/>
+      <c r="J14" s="82" t="n"/>
+      <c r="K14" s="82" t="n"/>
+      <c r="L14" s="82" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1" s="36">
       <c r="A15" s="70" t="inlineStr">
@@ -5258,30 +5290,30 @@
       <c r="H15" s="74" t="n"/>
       <c r="I15" s="70" t="n"/>
       <c r="J15" s="70" t="n"/>
-      <c r="K15" s="71" t="n"/>
-      <c r="L15" s="71" t="n"/>
+      <c r="K15" s="70" t="n"/>
+      <c r="L15" s="70" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1" s="36">
-      <c r="A16" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B16" s="72" t="inlineStr">
+      <c r="A16" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B16" s="82" t="inlineStr">
         <is>
           <t>Karl</t>
         </is>
       </c>
-      <c r="C16" s="73" t="n"/>
-      <c r="D16" s="73" t="n"/>
-      <c r="E16" s="73" t="n"/>
-      <c r="F16" s="73" t="n"/>
-      <c r="G16" s="73" t="n"/>
-      <c r="H16" s="73" t="n"/>
-      <c r="I16" s="72" t="n"/>
-      <c r="J16" s="72" t="n"/>
-      <c r="K16" s="71" t="n"/>
-      <c r="L16" s="71" t="n"/>
+      <c r="C16" s="83" t="n"/>
+      <c r="D16" s="83" t="n"/>
+      <c r="E16" s="83" t="n"/>
+      <c r="F16" s="83" t="n"/>
+      <c r="G16" s="83" t="n"/>
+      <c r="H16" s="83" t="n"/>
+      <c r="I16" s="82" t="n"/>
+      <c r="J16" s="82" t="n"/>
+      <c r="K16" s="82" t="n"/>
+      <c r="L16" s="82" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1" s="36">
       <c r="A17" s="70" t="inlineStr">
@@ -5302,30 +5334,30 @@
       <c r="H17" s="74" t="n"/>
       <c r="I17" s="70" t="n"/>
       <c r="J17" s="70" t="n"/>
-      <c r="K17" s="71" t="n"/>
-      <c r="L17" s="71" t="n"/>
+      <c r="K17" s="70" t="n"/>
+      <c r="L17" s="70" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1" s="36">
-      <c r="A18" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B18" s="72" t="inlineStr">
+      <c r="A18" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B18" s="82" t="inlineStr">
         <is>
           <t>Mike</t>
         </is>
       </c>
-      <c r="C18" s="73" t="n"/>
-      <c r="D18" s="73" t="n"/>
-      <c r="E18" s="73" t="n"/>
-      <c r="F18" s="73" t="n"/>
-      <c r="G18" s="73" t="n"/>
-      <c r="H18" s="73" t="n"/>
-      <c r="I18" s="72" t="n"/>
-      <c r="J18" s="72" t="n"/>
-      <c r="K18" s="71" t="n"/>
-      <c r="L18" s="71" t="n"/>
+      <c r="C18" s="83" t="n"/>
+      <c r="D18" s="83" t="n"/>
+      <c r="E18" s="83" t="n"/>
+      <c r="F18" s="83" t="n"/>
+      <c r="G18" s="83" t="n"/>
+      <c r="H18" s="83" t="n"/>
+      <c r="I18" s="82" t="n"/>
+      <c r="J18" s="82" t="n"/>
+      <c r="K18" s="82" t="n"/>
+      <c r="L18" s="82" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1" s="36">
       <c r="A19" s="70" t="inlineStr">
@@ -5346,30 +5378,30 @@
       <c r="H19" s="74" t="n"/>
       <c r="I19" s="70" t="n"/>
       <c r="J19" s="70" t="n"/>
-      <c r="K19" s="71" t="n"/>
-      <c r="L19" s="71" t="n"/>
+      <c r="K19" s="70" t="n"/>
+      <c r="L19" s="70" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1" s="36">
-      <c r="A20" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B20" s="72" t="inlineStr">
+      <c r="A20" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B20" s="82" t="inlineStr">
         <is>
           <t>Zabby</t>
         </is>
       </c>
-      <c r="C20" s="73" t="n"/>
-      <c r="D20" s="73" t="n"/>
-      <c r="E20" s="73" t="n"/>
-      <c r="F20" s="73" t="n"/>
-      <c r="G20" s="73" t="n"/>
-      <c r="H20" s="73" t="n"/>
-      <c r="I20" s="72" t="n"/>
-      <c r="J20" s="72" t="n"/>
-      <c r="K20" s="71" t="n"/>
-      <c r="L20" s="71" t="n"/>
+      <c r="C20" s="83" t="n"/>
+      <c r="D20" s="83" t="n"/>
+      <c r="E20" s="83" t="n"/>
+      <c r="F20" s="83" t="n"/>
+      <c r="G20" s="83" t="n"/>
+      <c r="H20" s="83" t="n"/>
+      <c r="I20" s="82" t="n"/>
+      <c r="J20" s="82" t="n"/>
+      <c r="K20" s="82" t="n"/>
+      <c r="L20" s="82" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1" s="36">
       <c r="A21" s="70" t="inlineStr">
@@ -5390,30 +5422,30 @@
       <c r="H21" s="74" t="n"/>
       <c r="I21" s="70" t="n"/>
       <c r="J21" s="70" t="n"/>
-      <c r="K21" s="71" t="n"/>
-      <c r="L21" s="71" t="n"/>
+      <c r="K21" s="70" t="n"/>
+      <c r="L21" s="70" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1" s="36">
-      <c r="A22" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B22" s="72" t="inlineStr">
+      <c r="A22" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B22" s="82" t="inlineStr">
         <is>
           <t>Eddy</t>
         </is>
       </c>
-      <c r="C22" s="73" t="n"/>
-      <c r="D22" s="73" t="n"/>
-      <c r="E22" s="73" t="n"/>
-      <c r="F22" s="73" t="n"/>
-      <c r="G22" s="73" t="n"/>
-      <c r="H22" s="73" t="n"/>
-      <c r="I22" s="72" t="n"/>
-      <c r="J22" s="72" t="n"/>
-      <c r="K22" s="71" t="n"/>
-      <c r="L22" s="71" t="n"/>
+      <c r="C22" s="83" t="n"/>
+      <c r="D22" s="83" t="n"/>
+      <c r="E22" s="83" t="n"/>
+      <c r="F22" s="83" t="n"/>
+      <c r="G22" s="83" t="n"/>
+      <c r="H22" s="83" t="n"/>
+      <c r="I22" s="82" t="n"/>
+      <c r="J22" s="82" t="n"/>
+      <c r="K22" s="82" t="n"/>
+      <c r="L22" s="82" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="36">
       <c r="A23" s="70" t="inlineStr">
@@ -5434,30 +5466,30 @@
       <c r="H23" s="74" t="n"/>
       <c r="I23" s="70" t="n"/>
       <c r="J23" s="70" t="n"/>
-      <c r="K23" s="71" t="n"/>
-      <c r="L23" s="71" t="n"/>
+      <c r="K23" s="70" t="n"/>
+      <c r="L23" s="70" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1" s="36">
-      <c r="A24" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B24" s="72" t="inlineStr">
+      <c r="A24" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B24" s="82" t="inlineStr">
         <is>
           <t>Barbara</t>
         </is>
       </c>
-      <c r="C24" s="73" t="n"/>
-      <c r="D24" s="73" t="n"/>
-      <c r="E24" s="73" t="n"/>
-      <c r="F24" s="73" t="n"/>
-      <c r="G24" s="73" t="n"/>
-      <c r="H24" s="73" t="n"/>
-      <c r="I24" s="72" t="n"/>
-      <c r="J24" s="72" t="n"/>
-      <c r="K24" s="71" t="n"/>
-      <c r="L24" s="71" t="n"/>
+      <c r="C24" s="83" t="n"/>
+      <c r="D24" s="83" t="n"/>
+      <c r="E24" s="83" t="n"/>
+      <c r="F24" s="83" t="n"/>
+      <c r="G24" s="83" t="n"/>
+      <c r="H24" s="83" t="n"/>
+      <c r="I24" s="82" t="n"/>
+      <c r="J24" s="82" t="n"/>
+      <c r="K24" s="82" t="n"/>
+      <c r="L24" s="82" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1" s="36">
       <c r="A25" s="70" t="inlineStr">
@@ -5478,30 +5510,30 @@
       <c r="H25" s="74" t="n"/>
       <c r="I25" s="70" t="n"/>
       <c r="J25" s="70" t="n"/>
-      <c r="K25" s="71" t="n"/>
-      <c r="L25" s="71" t="n"/>
+      <c r="K25" s="70" t="n"/>
+      <c r="L25" s="70" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="36">
-      <c r="A26" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B26" s="72" t="inlineStr">
+      <c r="A26" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B26" s="82" t="inlineStr">
         <is>
           <t>Calvin</t>
         </is>
       </c>
-      <c r="C26" s="73" t="n"/>
-      <c r="D26" s="73" t="n"/>
-      <c r="E26" s="73" t="n"/>
-      <c r="F26" s="73" t="n"/>
-      <c r="G26" s="73" t="n"/>
-      <c r="H26" s="73" t="n"/>
-      <c r="I26" s="72" t="n"/>
-      <c r="J26" s="72" t="n"/>
-      <c r="K26" s="71" t="n"/>
-      <c r="L26" s="71" t="n"/>
+      <c r="C26" s="83" t="n"/>
+      <c r="D26" s="83" t="n"/>
+      <c r="E26" s="83" t="n"/>
+      <c r="F26" s="83" t="n"/>
+      <c r="G26" s="83" t="n"/>
+      <c r="H26" s="83" t="n"/>
+      <c r="I26" s="82" t="n"/>
+      <c r="J26" s="82" t="n"/>
+      <c r="K26" s="82" t="n"/>
+      <c r="L26" s="82" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1" s="36">
       <c r="A27" s="70" t="inlineStr">
@@ -5522,30 +5554,30 @@
       <c r="H27" s="74" t="n"/>
       <c r="I27" s="70" t="n"/>
       <c r="J27" s="70" t="n"/>
-      <c r="K27" s="71" t="n"/>
-      <c r="L27" s="71" t="n"/>
+      <c r="K27" s="70" t="n"/>
+      <c r="L27" s="70" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1" s="36">
-      <c r="A28" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B28" s="72" t="inlineStr">
+      <c r="A28" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B28" s="82" t="inlineStr">
         <is>
           <t>Demi</t>
         </is>
       </c>
-      <c r="C28" s="73" t="n"/>
-      <c r="D28" s="73" t="n"/>
-      <c r="E28" s="73" t="n"/>
-      <c r="F28" s="73" t="n"/>
-      <c r="G28" s="73" t="n"/>
-      <c r="H28" s="73" t="n"/>
-      <c r="I28" s="72" t="n"/>
-      <c r="J28" s="72" t="n"/>
-      <c r="K28" s="71" t="n"/>
-      <c r="L28" s="71" t="n"/>
+      <c r="C28" s="83" t="n"/>
+      <c r="D28" s="83" t="n"/>
+      <c r="E28" s="83" t="n"/>
+      <c r="F28" s="83" t="n"/>
+      <c r="G28" s="83" t="n"/>
+      <c r="H28" s="83" t="n"/>
+      <c r="I28" s="82" t="n"/>
+      <c r="J28" s="82" t="n"/>
+      <c r="K28" s="82" t="n"/>
+      <c r="L28" s="82" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1" s="36">
       <c r="A29" s="70" t="inlineStr">
@@ -5566,30 +5598,30 @@
       <c r="H29" s="74" t="n"/>
       <c r="I29" s="70" t="n"/>
       <c r="J29" s="70" t="n"/>
-      <c r="K29" s="71" t="n"/>
-      <c r="L29" s="71" t="n"/>
+      <c r="K29" s="70" t="n"/>
+      <c r="L29" s="70" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1" s="36">
-      <c r="A30" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B30" s="72" t="inlineStr">
+      <c r="A30" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B30" s="82" t="inlineStr">
         <is>
           <t>Edgar</t>
         </is>
       </c>
-      <c r="C30" s="73" t="n"/>
-      <c r="D30" s="73" t="n"/>
-      <c r="E30" s="73" t="n"/>
-      <c r="F30" s="73" t="n"/>
-      <c r="G30" s="73" t="n"/>
-      <c r="H30" s="73" t="n"/>
-      <c r="I30" s="72" t="n"/>
-      <c r="J30" s="72" t="n"/>
-      <c r="K30" s="71" t="n"/>
-      <c r="L30" s="71" t="n"/>
+      <c r="C30" s="83" t="n"/>
+      <c r="D30" s="83" t="n"/>
+      <c r="E30" s="83" t="n"/>
+      <c r="F30" s="83" t="n"/>
+      <c r="G30" s="83" t="n"/>
+      <c r="H30" s="83" t="n"/>
+      <c r="I30" s="82" t="n"/>
+      <c r="J30" s="82" t="n"/>
+      <c r="K30" s="82" t="n"/>
+      <c r="L30" s="82" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1" s="36">
       <c r="A31" s="70" t="inlineStr">
@@ -5610,30 +5642,30 @@
       <c r="H31" s="74" t="n"/>
       <c r="I31" s="70" t="n"/>
       <c r="J31" s="70" t="n"/>
-      <c r="K31" s="71" t="n"/>
-      <c r="L31" s="71" t="n"/>
+      <c r="K31" s="70" t="n"/>
+      <c r="L31" s="70" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1" s="36">
-      <c r="A32" s="72" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B32" s="72" t="inlineStr">
+      <c r="A32" s="82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B32" s="82" t="inlineStr">
         <is>
           <t>Felicity</t>
         </is>
       </c>
-      <c r="C32" s="73" t="n"/>
-      <c r="D32" s="73" t="n"/>
-      <c r="E32" s="73" t="n"/>
-      <c r="F32" s="73" t="n"/>
-      <c r="G32" s="73" t="n"/>
-      <c r="H32" s="73" t="n"/>
-      <c r="I32" s="72" t="n"/>
-      <c r="J32" s="72" t="n"/>
-      <c r="K32" s="71" t="n"/>
-      <c r="L32" s="71" t="n"/>
+      <c r="C32" s="83" t="n"/>
+      <c r="D32" s="83" t="n"/>
+      <c r="E32" s="83" t="n"/>
+      <c r="F32" s="83" t="n"/>
+      <c r="G32" s="83" t="n"/>
+      <c r="H32" s="83" t="n"/>
+      <c r="I32" s="82" t="n"/>
+      <c r="J32" s="82" t="n"/>
+      <c r="K32" s="82" t="n"/>
+      <c r="L32" s="82" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1" s="36">
       <c r="A33" s="70" t="inlineStr">
@@ -5654,26 +5686,26 @@
       <c r="H33" s="74" t="n"/>
       <c r="I33" s="70" t="n"/>
       <c r="J33" s="70" t="n"/>
-      <c r="K33" s="71" t="n"/>
-      <c r="L33" s="71" t="n"/>
+      <c r="K33" s="70" t="n"/>
+      <c r="L33" s="70" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1" s="36">
-      <c r="A34" s="75" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B34" s="76" t="n"/>
-      <c r="C34" s="76" t="n"/>
-      <c r="D34" s="76" t="n"/>
-      <c r="E34" s="76" t="n"/>
-      <c r="F34" s="76" t="n"/>
-      <c r="G34" s="76" t="n"/>
-      <c r="H34" s="75" t="n"/>
-      <c r="I34" s="72" t="n"/>
-      <c r="J34" s="72" t="n"/>
-      <c r="K34" s="71" t="n"/>
-      <c r="L34" s="71" t="n"/>
+      <c r="A34" s="84" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B34" s="85" t="n"/>
+      <c r="C34" s="85" t="n"/>
+      <c r="D34" s="85" t="n"/>
+      <c r="E34" s="85" t="n"/>
+      <c r="F34" s="85" t="n"/>
+      <c r="G34" s="85" t="n"/>
+      <c r="H34" s="84" t="n"/>
+      <c r="I34" s="82" t="n"/>
+      <c r="J34" s="82" t="n"/>
+      <c r="K34" s="82" t="n"/>
+      <c r="L34" s="82" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1" s="36">
       <c r="A35" s="67" t="inlineStr">
@@ -5688,39 +5720,39 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="69" t="n"/>
-      <c r="C36" s="69" t="n"/>
-      <c r="D36" s="69" t="n"/>
-      <c r="E36" s="69" t="n"/>
-      <c r="F36" s="69" t="n"/>
-      <c r="G36" s="69" t="n"/>
-      <c r="H36" s="68" t="n"/>
+      <c r="B36" s="80" t="n"/>
+      <c r="C36" s="80" t="n"/>
+      <c r="D36" s="80" t="n"/>
+      <c r="E36" s="80" t="n"/>
+      <c r="F36" s="80" t="n"/>
+      <c r="G36" s="80" t="n"/>
+      <c r="H36" s="81" t="n"/>
       <c r="I36" s="70" t="n"/>
       <c r="J36" s="70" t="n"/>
-      <c r="K36" s="71" t="n"/>
-      <c r="L36" s="71" t="n"/>
+      <c r="K36" s="70" t="n"/>
+      <c r="L36" s="70" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="36">
-      <c r="A37" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B37" s="72" t="inlineStr">
+      <c r="A37" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B37" s="82" t="inlineStr">
         <is>
           <t>Marco</t>
         </is>
       </c>
-      <c r="C37" s="73" t="n"/>
-      <c r="D37" s="73" t="n"/>
-      <c r="E37" s="73" t="n"/>
-      <c r="F37" s="73" t="n"/>
-      <c r="G37" s="73" t="n"/>
-      <c r="H37" s="73" t="n"/>
-      <c r="I37" s="72" t="n"/>
-      <c r="J37" s="72" t="n"/>
-      <c r="K37" s="71" t="n"/>
-      <c r="L37" s="71" t="n"/>
+      <c r="C37" s="83" t="n"/>
+      <c r="D37" s="83" t="n"/>
+      <c r="E37" s="83" t="n"/>
+      <c r="F37" s="83" t="n"/>
+      <c r="G37" s="83" t="n"/>
+      <c r="H37" s="83" t="n"/>
+      <c r="I37" s="82" t="n"/>
+      <c r="J37" s="82" t="n"/>
+      <c r="K37" s="82" t="n"/>
+      <c r="L37" s="82" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1" s="36">
       <c r="A38" s="70" t="inlineStr">
@@ -5741,30 +5773,30 @@
       <c r="H38" s="74" t="n"/>
       <c r="I38" s="70" t="n"/>
       <c r="J38" s="70" t="n"/>
-      <c r="K38" s="71" t="n"/>
-      <c r="L38" s="71" t="n"/>
+      <c r="K38" s="70" t="n"/>
+      <c r="L38" s="70" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1" s="36">
-      <c r="A39" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B39" s="72" t="inlineStr">
+      <c r="A39" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B39" s="82" t="inlineStr">
         <is>
           <t>Marcus</t>
         </is>
       </c>
-      <c r="C39" s="73" t="n"/>
-      <c r="D39" s="73" t="n"/>
-      <c r="E39" s="73" t="n"/>
-      <c r="F39" s="73" t="n"/>
-      <c r="G39" s="73" t="n"/>
-      <c r="H39" s="73" t="n"/>
-      <c r="I39" s="72" t="n"/>
-      <c r="J39" s="72" t="n"/>
-      <c r="K39" s="71" t="n"/>
-      <c r="L39" s="71" t="n"/>
+      <c r="C39" s="83" t="n"/>
+      <c r="D39" s="83" t="n"/>
+      <c r="E39" s="83" t="n"/>
+      <c r="F39" s="83" t="n"/>
+      <c r="G39" s="83" t="n"/>
+      <c r="H39" s="83" t="n"/>
+      <c r="I39" s="82" t="n"/>
+      <c r="J39" s="82" t="n"/>
+      <c r="K39" s="82" t="n"/>
+      <c r="L39" s="82" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="36">
       <c r="A40" s="70" t="inlineStr">
@@ -5785,30 +5817,30 @@
       <c r="H40" s="74" t="n"/>
       <c r="I40" s="70" t="n"/>
       <c r="J40" s="70" t="n"/>
-      <c r="K40" s="71" t="n"/>
-      <c r="L40" s="71" t="n"/>
+      <c r="K40" s="70" t="n"/>
+      <c r="L40" s="70" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1" s="36">
-      <c r="A41" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B41" s="72" t="inlineStr">
+      <c r="A41" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B41" s="82" t="inlineStr">
         <is>
           <t>Amy</t>
         </is>
       </c>
-      <c r="C41" s="73" t="n"/>
-      <c r="D41" s="73" t="n"/>
-      <c r="E41" s="73" t="n"/>
-      <c r="F41" s="73" t="n"/>
-      <c r="G41" s="73" t="n"/>
-      <c r="H41" s="73" t="n"/>
-      <c r="I41" s="72" t="n"/>
-      <c r="J41" s="72" t="n"/>
-      <c r="K41" s="71" t="n"/>
-      <c r="L41" s="71" t="n"/>
+      <c r="C41" s="83" t="n"/>
+      <c r="D41" s="83" t="n"/>
+      <c r="E41" s="83" t="n"/>
+      <c r="F41" s="83" t="n"/>
+      <c r="G41" s="83" t="n"/>
+      <c r="H41" s="83" t="n"/>
+      <c r="I41" s="82" t="n"/>
+      <c r="J41" s="82" t="n"/>
+      <c r="K41" s="82" t="n"/>
+      <c r="L41" s="82" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1" s="36">
       <c r="A42" s="70" t="inlineStr">
@@ -5829,30 +5861,30 @@
       <c r="H42" s="74" t="n"/>
       <c r="I42" s="70" t="n"/>
       <c r="J42" s="70" t="n"/>
-      <c r="K42" s="71" t="n"/>
-      <c r="L42" s="71" t="n"/>
+      <c r="K42" s="70" t="n"/>
+      <c r="L42" s="70" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1" s="36">
-      <c r="A43" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B43" s="72" t="inlineStr">
+      <c r="A43" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B43" s="82" t="inlineStr">
         <is>
           <t>Irma</t>
         </is>
       </c>
-      <c r="C43" s="73" t="n"/>
-      <c r="D43" s="73" t="n"/>
-      <c r="E43" s="73" t="n"/>
-      <c r="F43" s="73" t="n"/>
-      <c r="G43" s="73" t="n"/>
-      <c r="H43" s="73" t="n"/>
-      <c r="I43" s="72" t="n"/>
-      <c r="J43" s="72" t="n"/>
-      <c r="K43" s="71" t="n"/>
-      <c r="L43" s="71" t="n"/>
+      <c r="C43" s="83" t="n"/>
+      <c r="D43" s="83" t="n"/>
+      <c r="E43" s="83" t="n"/>
+      <c r="F43" s="83" t="n"/>
+      <c r="G43" s="83" t="n"/>
+      <c r="H43" s="83" t="n"/>
+      <c r="I43" s="82" t="n"/>
+      <c r="J43" s="82" t="n"/>
+      <c r="K43" s="82" t="n"/>
+      <c r="L43" s="82" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1" s="36">
       <c r="A44" s="70" t="inlineStr">
@@ -5873,30 +5905,30 @@
       <c r="H44" s="74" t="n"/>
       <c r="I44" s="70" t="n"/>
       <c r="J44" s="70" t="n"/>
-      <c r="K44" s="71" t="n"/>
-      <c r="L44" s="71" t="n"/>
+      <c r="K44" s="70" t="n"/>
+      <c r="L44" s="70" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1" s="36">
-      <c r="A45" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B45" s="72" t="inlineStr">
+      <c r="A45" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B45" s="82" t="inlineStr">
         <is>
           <t>Bruno</t>
         </is>
       </c>
-      <c r="C45" s="73" t="n"/>
-      <c r="D45" s="73" t="n"/>
-      <c r="E45" s="73" t="n"/>
-      <c r="F45" s="73" t="n"/>
-      <c r="G45" s="73" t="n"/>
-      <c r="H45" s="73" t="n"/>
-      <c r="I45" s="72" t="n"/>
-      <c r="J45" s="72" t="n"/>
-      <c r="K45" s="71" t="n"/>
-      <c r="L45" s="71" t="n"/>
+      <c r="C45" s="83" t="n"/>
+      <c r="D45" s="83" t="n"/>
+      <c r="E45" s="83" t="n"/>
+      <c r="F45" s="83" t="n"/>
+      <c r="G45" s="83" t="n"/>
+      <c r="H45" s="83" t="n"/>
+      <c r="I45" s="82" t="n"/>
+      <c r="J45" s="82" t="n"/>
+      <c r="K45" s="82" t="n"/>
+      <c r="L45" s="82" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1" s="36">
       <c r="A46" s="70" t="inlineStr">
@@ -5917,30 +5949,30 @@
       <c r="H46" s="74" t="n"/>
       <c r="I46" s="70" t="n"/>
       <c r="J46" s="70" t="n"/>
-      <c r="K46" s="71" t="n"/>
-      <c r="L46" s="71" t="n"/>
+      <c r="K46" s="70" t="n"/>
+      <c r="L46" s="70" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="36">
-      <c r="A47" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B47" s="72" t="inlineStr">
+      <c r="A47" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B47" s="82" t="inlineStr">
         <is>
           <t>Shana</t>
         </is>
       </c>
-      <c r="C47" s="73" t="n"/>
-      <c r="D47" s="73" t="n"/>
-      <c r="E47" s="73" t="n"/>
-      <c r="F47" s="73" t="n"/>
-      <c r="G47" s="73" t="n"/>
-      <c r="H47" s="73" t="n"/>
-      <c r="I47" s="72" t="n"/>
-      <c r="J47" s="72" t="n"/>
-      <c r="K47" s="71" t="n"/>
-      <c r="L47" s="71" t="n"/>
+      <c r="C47" s="83" t="n"/>
+      <c r="D47" s="83" t="n"/>
+      <c r="E47" s="83" t="n"/>
+      <c r="F47" s="83" t="n"/>
+      <c r="G47" s="83" t="n"/>
+      <c r="H47" s="83" t="n"/>
+      <c r="I47" s="82" t="n"/>
+      <c r="J47" s="82" t="n"/>
+      <c r="K47" s="82" t="n"/>
+      <c r="L47" s="82" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1" s="36">
       <c r="A48" s="70" t="inlineStr">
@@ -5961,30 +5993,30 @@
       <c r="H48" s="74" t="n"/>
       <c r="I48" s="70" t="n"/>
       <c r="J48" s="70" t="n"/>
-      <c r="K48" s="71" t="n"/>
-      <c r="L48" s="71" t="n"/>
+      <c r="K48" s="70" t="n"/>
+      <c r="L48" s="70" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1" s="36">
-      <c r="A49" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B49" s="72" t="inlineStr">
+      <c r="A49" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B49" s="82" t="inlineStr">
         <is>
           <t>Helena</t>
         </is>
       </c>
-      <c r="C49" s="73" t="n"/>
-      <c r="D49" s="73" t="n"/>
-      <c r="E49" s="73" t="n"/>
-      <c r="F49" s="73" t="n"/>
-      <c r="G49" s="73" t="n"/>
-      <c r="H49" s="73" t="n"/>
-      <c r="I49" s="72" t="n"/>
-      <c r="J49" s="72" t="n"/>
-      <c r="K49" s="71" t="n"/>
-      <c r="L49" s="71" t="n"/>
+      <c r="C49" s="83" t="n"/>
+      <c r="D49" s="83" t="n"/>
+      <c r="E49" s="83" t="n"/>
+      <c r="F49" s="83" t="n"/>
+      <c r="G49" s="83" t="n"/>
+      <c r="H49" s="83" t="n"/>
+      <c r="I49" s="82" t="n"/>
+      <c r="J49" s="82" t="n"/>
+      <c r="K49" s="82" t="n"/>
+      <c r="L49" s="82" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="36">
       <c r="A50" s="70" t="inlineStr">
@@ -6005,30 +6037,30 @@
       <c r="H50" s="74" t="n"/>
       <c r="I50" s="70" t="n"/>
       <c r="J50" s="70" t="n"/>
-      <c r="K50" s="71" t="n"/>
-      <c r="L50" s="71" t="n"/>
+      <c r="K50" s="70" t="n"/>
+      <c r="L50" s="70" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1" s="36">
-      <c r="A51" s="72" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B51" s="72" t="inlineStr">
+      <c r="A51" s="82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B51" s="82" t="inlineStr">
         <is>
           <t>Ulysses</t>
         </is>
       </c>
-      <c r="C51" s="73" t="n"/>
-      <c r="D51" s="73" t="n"/>
-      <c r="E51" s="73" t="n"/>
-      <c r="F51" s="73" t="n"/>
-      <c r="G51" s="73" t="n"/>
-      <c r="H51" s="73" t="n"/>
-      <c r="I51" s="72" t="n"/>
-      <c r="J51" s="72" t="n"/>
-      <c r="K51" s="71" t="n"/>
-      <c r="L51" s="71" t="n"/>
+      <c r="C51" s="83" t="n"/>
+      <c r="D51" s="83" t="n"/>
+      <c r="E51" s="83" t="n"/>
+      <c r="F51" s="83" t="n"/>
+      <c r="G51" s="83" t="n"/>
+      <c r="H51" s="83" t="n"/>
+      <c r="I51" s="82" t="n"/>
+      <c r="J51" s="82" t="n"/>
+      <c r="K51" s="82" t="n"/>
+      <c r="L51" s="82" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="48" t="inlineStr">

</xml_diff>

<commit_message>
All sheets: Blank numbering in row 3, title+description in row 54, full formatting
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -173,6 +173,11 @@
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="26">
@@ -417,7 +422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -661,6 +666,9 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1517,145 +1525,145 @@
       </c>
       <c r="C3" s="82" t="inlineStr">
         <is>
-          <t>A1
+          <t>Blank 1
 Prior belief</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
-          <t>A2
+          <t>Blank 2
 Data-based exploration</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>A3
+          <t>Blank 3
 Meaningful difference found</t>
         </is>
       </c>
       <c r="F3" s="82" t="inlineStr">
         <is>
-          <t>A4
+          <t>Blank 4
 First variable justification</t>
         </is>
       </c>
       <c r="G3" s="82" t="inlineStr">
         <is>
-          <t>B1
+          <t>Blank 5
 Tree 1 — build + EMIT</t>
         </is>
       </c>
       <c r="H3" s="82" t="inlineStr">
         <is>
-          <t>B2
+          <t>Blank 6
 Tree 2 — build + EMIT</t>
         </is>
       </c>
       <c r="I3" s="82" t="inlineStr">
         <is>
-          <t>B3
+          <t>Blank 7
 Tree 3 — build + EMIT</t>
         </is>
       </c>
       <c r="J3" s="82" t="inlineStr">
         <is>
-          <t>B4
+          <t>Blank 8
 Best tree + criteria</t>
         </is>
       </c>
       <c r="K3" s="82" t="inlineStr">
         <is>
-          <t>C1
+          <t>Blank 9
 Threshold optimization</t>
         </is>
       </c>
       <c r="L3" s="82" t="inlineStr">
         <is>
-          <t>C2
+          <t>Blank 10
 Threshold effect</t>
         </is>
       </c>
       <c r="M3" s="82" t="inlineStr">
         <is>
-          <t>C3
+          <t>Blank 11
 Best threshold + reasoning</t>
         </is>
       </c>
       <c r="N3" s="82" t="inlineStr">
         <is>
-          <t>D1
+          <t>Blank 12
 Two-level tree — build + EMIT</t>
         </is>
       </c>
       <c r="O3" s="82" t="inlineStr">
         <is>
-          <t>D2
+          <t>Blank 13
 Second level effect</t>
         </is>
       </c>
       <c r="P3" s="82" t="inlineStr">
         <is>
-          <t>D3
+          <t>Blank 14
 Best variable combination</t>
         </is>
       </c>
       <c r="Q3" s="82" t="inlineStr">
         <is>
-          <t>D4
+          <t>Blank 15
 Stopping criterion</t>
         </is>
       </c>
       <c r="R3" s="82" t="inlineStr">
         <is>
-          <t>E
+          <t>Blank 16
 Metrics</t>
         </is>
       </c>
       <c r="S3" s="82" t="inlineStr">
         <is>
-          <t>E1
+          <t>Blank 17
 Metric interpretation</t>
         </is>
       </c>
       <c r="T3" s="82" t="inlineStr">
         <is>
-          <t>E2
+          <t>Blank 18
 Error type analysis</t>
         </is>
       </c>
       <c r="U3" s="82" t="inlineStr">
         <is>
-          <t>E3
+          <t>Blank 19
 Good-enough criterion</t>
         </is>
       </c>
       <c r="V3" s="82" t="inlineStr">
         <is>
-          <t>E4
+          <t>Blank 20
 Perfect classification</t>
         </is>
       </c>
       <c r="W3" s="82" t="inlineStr">
         <is>
-          <t>F1
+          <t>Blank 21
 Test set application</t>
         </is>
       </c>
       <c r="X3" s="82" t="inlineStr">
         <is>
-          <t>F2
+          <t>Blank 22
 Train vs test comparison</t>
         </is>
       </c>
       <c r="Y3" s="82" t="inlineStr">
         <is>
-          <t>G1
+          <t>Blank 23
 What the model learned</t>
         </is>
       </c>
       <c r="Z3" s="82" t="inlineStr">
         <is>
-          <t>G2
+          <t>Blank 24
 Personal reflection</t>
         </is>
       </c>
@@ -1683,33 +1691,33 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
-      <c r="L5" s="84" t="n"/>
-      <c r="M5" s="84" t="n"/>
-      <c r="N5" s="84" t="n"/>
-      <c r="O5" s="84" t="n"/>
-      <c r="P5" s="84" t="n"/>
-      <c r="Q5" s="84" t="n"/>
-      <c r="R5" s="84" t="n"/>
-      <c r="S5" s="84" t="n"/>
-      <c r="T5" s="84" t="n"/>
-      <c r="U5" s="84" t="n"/>
-      <c r="V5" s="84" t="n"/>
-      <c r="W5" s="84" t="n"/>
-      <c r="X5" s="84" t="n"/>
-      <c r="Y5" s="84" t="n"/>
-      <c r="Z5" s="84" t="n"/>
-      <c r="AA5" s="84" t="n"/>
-      <c r="AB5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="86" t="n"/>
+      <c r="L5" s="86" t="n"/>
+      <c r="M5" s="86" t="n"/>
+      <c r="N5" s="86" t="n"/>
+      <c r="O5" s="86" t="n"/>
+      <c r="P5" s="86" t="n"/>
+      <c r="Q5" s="86" t="n"/>
+      <c r="R5" s="86" t="n"/>
+      <c r="S5" s="86" t="n"/>
+      <c r="T5" s="86" t="n"/>
+      <c r="U5" s="86" t="n"/>
+      <c r="V5" s="86" t="n"/>
+      <c r="W5" s="86" t="n"/>
+      <c r="X5" s="86" t="n"/>
+      <c r="Y5" s="86" t="n"/>
+      <c r="Z5" s="86" t="n"/>
+      <c r="AA5" s="86" t="n"/>
+      <c r="AB5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -2822,33 +2830,33 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
-      <c r="L36" s="84" t="n"/>
-      <c r="M36" s="84" t="n"/>
-      <c r="N36" s="84" t="n"/>
-      <c r="O36" s="84" t="n"/>
-      <c r="P36" s="84" t="n"/>
-      <c r="Q36" s="84" t="n"/>
-      <c r="R36" s="84" t="n"/>
-      <c r="S36" s="84" t="n"/>
-      <c r="T36" s="84" t="n"/>
-      <c r="U36" s="84" t="n"/>
-      <c r="V36" s="84" t="n"/>
-      <c r="W36" s="84" t="n"/>
-      <c r="X36" s="84" t="n"/>
-      <c r="Y36" s="84" t="n"/>
-      <c r="Z36" s="84" t="n"/>
-      <c r="AA36" s="84" t="n"/>
-      <c r="AB36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="86" t="n"/>
+      <c r="L36" s="86" t="n"/>
+      <c r="M36" s="86" t="n"/>
+      <c r="N36" s="86" t="n"/>
+      <c r="O36" s="86" t="n"/>
+      <c r="P36" s="86" t="n"/>
+      <c r="Q36" s="86" t="n"/>
+      <c r="R36" s="86" t="n"/>
+      <c r="S36" s="86" t="n"/>
+      <c r="T36" s="86" t="n"/>
+      <c r="U36" s="86" t="n"/>
+      <c r="V36" s="86" t="n"/>
+      <c r="W36" s="86" t="n"/>
+      <c r="X36" s="86" t="n"/>
+      <c r="Y36" s="86" t="n"/>
+      <c r="Z36" s="86" t="n"/>
+      <c r="AA36" s="86" t="n"/>
+      <c r="AB36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -3420,40 +3428,39 @@
       <c r="AA51" s="85" t="n"/>
       <c r="AB51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
-      <c r="H53" s="84" t="n"/>
-      <c r="I53" s="84" t="n"/>
-      <c r="J53" s="84" t="n"/>
-      <c r="K53" s="84" t="n"/>
-      <c r="L53" s="84" t="n"/>
-      <c r="M53" s="84" t="n"/>
-      <c r="N53" s="84" t="n"/>
-      <c r="O53" s="84" t="n"/>
-      <c r="P53" s="84" t="n"/>
-      <c r="Q53" s="84" t="n"/>
-      <c r="R53" s="84" t="n"/>
-      <c r="S53" s="84" t="n"/>
-      <c r="T53" s="84" t="n"/>
-      <c r="U53" s="84" t="n"/>
-      <c r="V53" s="84" t="n"/>
-      <c r="W53" s="84" t="n"/>
-      <c r="X53" s="84" t="n"/>
-      <c r="Y53" s="84" t="n"/>
-      <c r="Z53" s="84" t="n"/>
-      <c r="AA53" s="84" t="n"/>
-      <c r="AB53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="86" t="n"/>
+      <c r="H53" s="86" t="n"/>
+      <c r="I53" s="86" t="n"/>
+      <c r="J53" s="86" t="n"/>
+      <c r="K53" s="86" t="n"/>
+      <c r="L53" s="86" t="n"/>
+      <c r="M53" s="86" t="n"/>
+      <c r="N53" s="86" t="n"/>
+      <c r="O53" s="86" t="n"/>
+      <c r="P53" s="86" t="n"/>
+      <c r="Q53" s="86" t="n"/>
+      <c r="R53" s="86" t="n"/>
+      <c r="S53" s="86" t="n"/>
+      <c r="T53" s="86" t="n"/>
+      <c r="U53" s="86" t="n"/>
+      <c r="V53" s="86" t="n"/>
+      <c r="W53" s="86" t="n"/>
+      <c r="X53" s="86" t="n"/>
+      <c r="Y53" s="86" t="n"/>
+      <c r="Z53" s="86" t="n"/>
+      <c r="AA53" s="86" t="n"/>
+      <c r="AB53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -3462,124 +3469,148 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>A1: Names variable(s) predicted to determine recommendability — based on intuition, any answer ok</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>A2: Names variable(s) based on data WITH graph/visualization evidence (not just intuition)</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>A3: Yes/No response AND references actual data to support the answer</t>
-        </is>
-      </c>
-      <c r="F54" s="85" t="inlineStr">
-        <is>
-          <t>A4: Justifies first-variable choice using data evidence (not general knowledge such as 'fat is unhealthy')</t>
-        </is>
-      </c>
-      <c r="G54" s="85" t="inlineStr">
-        <is>
-          <t>B1: Builds single-level tree with one variable, records EMIT accuracy result</t>
-        </is>
-      </c>
-      <c r="H54" s="85" t="inlineStr">
-        <is>
-          <t>B2: Builds second single-level tree with a different variable, records EMIT</t>
-        </is>
-      </c>
-      <c r="I54" s="85" t="inlineStr">
-        <is>
-          <t>B3: Builds third single-level tree with yet another variable, records EMIT</t>
-        </is>
-      </c>
-      <c r="J54" s="85" t="inlineStr">
-        <is>
-          <t>B4: Identifies best tree among B1-B3 AND lists criteria used for comparison</t>
-        </is>
-      </c>
-      <c r="K54" s="85" t="inlineStr">
-        <is>
-          <t>C1: Tries different threshold values for best variable from B; saves best with EMIT</t>
-        </is>
-      </c>
-      <c r="L54" s="85" t="inlineStr">
-        <is>
-          <t>C2: Explains how changing the threshold value affects decision tree performance</t>
-        </is>
-      </c>
-      <c r="M54" s="85" t="inlineStr">
-        <is>
-          <t>C3: Identifies best threshold and explains how that conclusion was reached</t>
-        </is>
-      </c>
-      <c r="N54" s="85" t="inlineStr">
-        <is>
-          <t>D1: Adds a second variable to create a two-level tree; saves with EMIT</t>
-        </is>
-      </c>
-      <c r="O54" s="85" t="inlineStr">
-        <is>
-          <t>D2: Explains whether and how the second variable improved classification</t>
-        </is>
-      </c>
-      <c r="P54" s="85" t="inlineStr">
-        <is>
-          <t>D3: States which variable combination produced the best result</t>
-        </is>
-      </c>
-      <c r="Q54" s="85" t="inlineStr">
-        <is>
-          <t>D4: Explains how they decided they had reached their best decision tree</t>
-        </is>
-      </c>
-      <c r="R54" s="85" t="inlineStr">
-        <is>
-          <t>E (intro): Records Sensitivity and MCR values from EMIT for the best tree</t>
-        </is>
-      </c>
-      <c r="S54" s="85" t="inlineStr">
-        <is>
-          <t>E1: Explains which metric matters more for this model's purpose and why</t>
-        </is>
-      </c>
-      <c r="T54" s="85" t="inlineStr">
-        <is>
-          <t>E2: Identifies whether the model made more false positives or false negatives</t>
-        </is>
-      </c>
-      <c r="U54" s="85" t="inlineStr">
-        <is>
-          <t>E3: Reflects on how software / they would decide when a tree is good enough</t>
-        </is>
-      </c>
-      <c r="V54" s="85" t="inlineStr">
-        <is>
-          <t>E4: Reflects on whether DTs can achieve zero error; gives a reasoned answer</t>
-        </is>
-      </c>
-      <c r="W54" s="85" t="inlineStr">
-        <is>
-          <t>F1: Applies best tree to test dataset, evaluates with EMIT, records result</t>
-        </is>
-      </c>
-      <c r="X54" s="85" t="inlineStr">
-        <is>
-          <t>F2: Compares test vs. training performance and explains any difference</t>
-        </is>
-      </c>
-      <c r="Y54" s="85" t="inlineStr">
-        <is>
-          <t>G1: Explains what the decision tree model 'learned' from the training data</t>
-        </is>
-      </c>
-      <c r="Z54" s="85" t="inlineStr">
-        <is>
-          <t>G2: Reflects on personal learning during the tree-building process</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Prior belief
+Names variable(s) predicted to determine recommendability — based on intuition, any answer ok</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>Data-based exploration
+Names variable(s) based on data WITH graph/visualization evidence (not just intuition)</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Meaningful difference found
+Yes/No response AND references actual data to support the answer</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>First variable justification
+Justifies first-variable choice using data evidence (not general knowledge such as 'fat is unhealthy')</t>
+        </is>
+      </c>
+      <c r="G54" s="90" t="inlineStr">
+        <is>
+          <t>Tree 1 — build + EMIT
+Builds single-level tree with one variable, records EMIT accuracy result</t>
+        </is>
+      </c>
+      <c r="H54" s="90" t="inlineStr">
+        <is>
+          <t>Tree 2 — build + EMIT
+Builds second single-level tree with a different variable, records EMIT</t>
+        </is>
+      </c>
+      <c r="I54" s="90" t="inlineStr">
+        <is>
+          <t>Tree 3 — build + EMIT
+Builds third single-level tree with yet another variable, records EMIT</t>
+        </is>
+      </c>
+      <c r="J54" s="90" t="inlineStr">
+        <is>
+          <t>Best tree + criteria
+Identifies best tree among B1-B3 AND lists criteria used for comparison</t>
+        </is>
+      </c>
+      <c r="K54" s="90" t="inlineStr">
+        <is>
+          <t>Threshold optimization
+Tries different threshold values for best variable from B; saves best with EMIT</t>
+        </is>
+      </c>
+      <c r="L54" s="90" t="inlineStr">
+        <is>
+          <t>Threshold effect
+Explains how changing the threshold value affects decision tree performance</t>
+        </is>
+      </c>
+      <c r="M54" s="90" t="inlineStr">
+        <is>
+          <t>Best threshold + reasoning
+Identifies best threshold and explains how that conclusion was reached</t>
+        </is>
+      </c>
+      <c r="N54" s="90" t="inlineStr">
+        <is>
+          <t>Two-level tree — build + EMIT
+Adds a second variable to create a two-level tree; saves with EMIT</t>
+        </is>
+      </c>
+      <c r="O54" s="90" t="inlineStr">
+        <is>
+          <t>Second level effect
+Explains whether and how the second variable improved classification</t>
+        </is>
+      </c>
+      <c r="P54" s="90" t="inlineStr">
+        <is>
+          <t>Best variable combination
+States which variable combination produced the best result</t>
+        </is>
+      </c>
+      <c r="Q54" s="90" t="inlineStr">
+        <is>
+          <t>Stopping criterion
+Explains how they decided they had reached their best decision tree</t>
+        </is>
+      </c>
+      <c r="R54" s="90" t="inlineStr">
+        <is>
+          <t>Metrics
+E (intro): Records Sensitivity and MCR values from EMIT for the best tree</t>
+        </is>
+      </c>
+      <c r="S54" s="90" t="inlineStr">
+        <is>
+          <t>Metric interpretation
+Explains which metric matters more for this model's purpose and why</t>
+        </is>
+      </c>
+      <c r="T54" s="90" t="inlineStr">
+        <is>
+          <t>Error type analysis
+Identifies whether the model made more false positives or false negatives</t>
+        </is>
+      </c>
+      <c r="U54" s="90" t="inlineStr">
+        <is>
+          <t>Good-enough criterion
+Reflects on how software / they would decide when a tree is good enough</t>
+        </is>
+      </c>
+      <c r="V54" s="90" t="inlineStr">
+        <is>
+          <t>Perfect classification
+Reflects on whether DTs can achieve zero error; gives a reasoned answer</t>
+        </is>
+      </c>
+      <c r="W54" s="90" t="inlineStr">
+        <is>
+          <t>Test set application
+Applies best tree to test dataset, evaluates with EMIT, records result</t>
+        </is>
+      </c>
+      <c r="X54" s="90" t="inlineStr">
+        <is>
+          <t>Train vs test comparison
+Compares test vs. training performance and explains any difference</t>
+        </is>
+      </c>
+      <c r="Y54" s="90" t="inlineStr">
+        <is>
+          <t>What the model learned
+Explains what the decision tree model 'learned' from the training data</t>
+        </is>
+      </c>
+      <c r="Z54" s="90" t="inlineStr">
+        <is>
+          <t>Personal reflection
+Reflects on personal learning during the tree-building process</t>
         </is>
       </c>
       <c r="AA54" s="85" t="inlineStr">
@@ -3735,78 +3766,67 @@
       <c r="C3" s="82" t="inlineStr">
         <is>
           <t>Blank 1
-Target Label
-Determining the final classification result (e.g., 'not recommendable')</t>
+Target Label</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
           <t>Blank 2
-Data Object
-Recognizing the fundamental data entity or item (e.g., 'Hazelnut Wafer')</t>
+Data Object</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
           <t>Blank 3
-Feature Name
-Identifying the name of the independent variable (e.g., 'Fat')</t>
+Feature Name</t>
         </is>
       </c>
       <c r="F3" s="82" t="inlineStr">
         <is>
           <t>Blank 4
-Feature Value
-Extracting the specific quantitative measurement for an attribute (e.g., '31.9 g')</t>
+Feature Value</t>
         </is>
       </c>
       <c r="G3" s="82" t="inlineStr">
         <is>
           <t>Blank 5
-Data Instance
-Comprehending that an item acts as a single row or data point in a dataset (e.g., 'Individual foods are called objects...')</t>
+Data Instance</t>
         </is>
       </c>
       <c r="H3" s="82" t="inlineStr">
         <is>
           <t>Blank 6
-Specific Object
-Mapping a concrete, real-world example to the concept of a data object (e.g., 'A hazelnut wafer is an object')</t>
+Specific Object</t>
         </is>
       </c>
       <c r="I3" s="82" t="inlineStr">
         <is>
           <t>Blank 7
-Feature Variable
-Understanding the structural attributes (columns) that describe the data (e.g., 'features are located in the left column')</t>
+Feature Variable</t>
         </is>
       </c>
       <c r="J3" s="82" t="inlineStr">
         <is>
           <t>Blank 8
-Feature Count
-Calculating the dimensionality or total number of variables in the dataset (e.g., 'there are 7 features')</t>
+Feature Count</t>
         </is>
       </c>
       <c r="K3" s="82" t="inlineStr">
         <is>
           <t>Blank 9
-Feature List
-Enumerating all the independent variables that can be extracted (e.g., 'Energy, Fat, Saturated Fat...')</t>
+Feature List</t>
         </is>
       </c>
       <c r="L3" s="82" t="inlineStr">
         <is>
           <t>Blank 10
-Instance Name
-Associating a specific data value (like 31.9 g) back to the specific object it belongs to (e.g., 'Hazelnut Wafer contains 31.9 g of fat')</t>
+Instance Name</t>
         </is>
       </c>
       <c r="M3" s="82" t="inlineStr">
         <is>
           <t>Blank 11
-Assigned Label
-Grasping that the target variable serves as the final decision or output for that specific item (e.g., 'given the note not recommendable as a label...')</t>
+Assigned Label</t>
         </is>
       </c>
       <c r="N3" s="82" t="inlineStr">
@@ -3833,20 +3853,20 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
-      <c r="L5" s="84" t="n"/>
-      <c r="M5" s="84" t="n"/>
-      <c r="N5" s="84" t="n"/>
-      <c r="O5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="86" t="n"/>
+      <c r="L5" s="86" t="n"/>
+      <c r="M5" s="86" t="n"/>
+      <c r="N5" s="86" t="n"/>
+      <c r="O5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -4582,20 +4602,20 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
-      <c r="L36" s="84" t="n"/>
-      <c r="M36" s="84" t="n"/>
-      <c r="N36" s="84" t="n"/>
-      <c r="O36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="86" t="n"/>
+      <c r="L36" s="86" t="n"/>
+      <c r="M36" s="86" t="n"/>
+      <c r="N36" s="86" t="n"/>
+      <c r="O36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -4972,27 +4992,26 @@
       <c r="N51" s="85" t="n"/>
       <c r="O51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
-      <c r="H53" s="84" t="n"/>
-      <c r="I53" s="84" t="n"/>
-      <c r="J53" s="84" t="n"/>
-      <c r="K53" s="84" t="n"/>
-      <c r="L53" s="84" t="n"/>
-      <c r="M53" s="84" t="n"/>
-      <c r="N53" s="84" t="n"/>
-      <c r="O53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="86" t="n"/>
+      <c r="H53" s="86" t="n"/>
+      <c r="I53" s="86" t="n"/>
+      <c r="J53" s="86" t="n"/>
+      <c r="K53" s="86" t="n"/>
+      <c r="L53" s="86" t="n"/>
+      <c r="M53" s="86" t="n"/>
+      <c r="N53" s="86" t="n"/>
+      <c r="O53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -5001,59 +5020,70 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>Diagram arrow pointing to food card name -&gt; 'label' (etiket)</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>Diagram arrow pointing to 'Findikli Gofret' card -&gt; 'object' (nesne)</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>Diagram arrow pointing to left column of card -&gt; 'feature / variable / characteristic'</t>
-        </is>
-      </c>
-      <c r="F54" s="85" t="inlineStr">
-        <is>
-          <t>Diagram arrow pointing to a numeric cell -&gt; 'value of the feature / characteristic'</t>
-        </is>
-      </c>
-      <c r="G54" s="85" t="inlineStr">
-        <is>
-          <t>Cloze: 'Individual foods are called ___' -&gt; object (nesne)</t>
-        </is>
-      </c>
-      <c r="H54" s="85" t="inlineStr">
-        <is>
-          <t>Cloze: 'Hazelnut wafer is a ___' -&gt; object (nesne)</t>
-        </is>
-      </c>
-      <c r="I54" s="85" t="inlineStr">
-        <is>
-          <t>Cloze: left-column names are called '___ / characteristic / variable'</t>
-        </is>
-      </c>
-      <c r="J54" s="85" t="inlineStr">
-        <is>
-          <t>Cloze: 'How many features? ___' -&gt; 7 (yedi / seven)</t>
-        </is>
-      </c>
-      <c r="K54" s="85" t="inlineStr">
-        <is>
-          <t>Cloze: student writes all feature names: Energy, Fat, Saturated Fat, Carbohydrates, Sugar, Protein, Salt</t>
-        </is>
-      </c>
-      <c r="L54" s="85" t="inlineStr">
-        <is>
-          <t>Cloze: 'For example ___ contains 31.9g fat' -&gt; Hazelnut Wafer (Findikli Gofret)</t>
-        </is>
-      </c>
-      <c r="M54" s="85" t="inlineStr">
-        <is>
-          <t>Cloze: 'Hazelnut wafer has been given ___ as label' -&gt; not recommended (tavsiye edilemez)</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Target Label
+Diagram arrow pointing to food card name → 'label' (etiket)</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>Data Object
+Diagram arrow pointing to 'Findikli Gofret' card → 'object' (nesne)</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Feature Name
+Diagram arrow pointing to left column of card → 'feature / variable / characteristic'</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>Feature Value
+Diagram arrow pointing to a numeric cell → 'value of the feature / characteristic'</t>
+        </is>
+      </c>
+      <c r="G54" s="90" t="inlineStr">
+        <is>
+          <t>Data Instance
+Cloze: 'Individual foods are called ___' → object (nesne)</t>
+        </is>
+      </c>
+      <c r="H54" s="90" t="inlineStr">
+        <is>
+          <t>Specific Object
+Cloze: 'Hazelnut wafer is a ___' → object (nesne)</t>
+        </is>
+      </c>
+      <c r="I54" s="90" t="inlineStr">
+        <is>
+          <t>Feature Variable
+Cloze: left-column names are called '___ / characteristic / variable'</t>
+        </is>
+      </c>
+      <c r="J54" s="90" t="inlineStr">
+        <is>
+          <t>Feature Count
+Cloze: 'How many features? ___' → 7 (yedi / seven)</t>
+        </is>
+      </c>
+      <c r="K54" s="90" t="inlineStr">
+        <is>
+          <t>Feature List
+Cloze: student writes all feature names: Energy, Fat, Saturated Fat, Carbohydrates, Sugar, Protein, Salt</t>
+        </is>
+      </c>
+      <c r="L54" s="90" t="inlineStr">
+        <is>
+          <t>Instance Name
+Cloze: 'For example ___ contains 31.9g fat' → Hazelnut Wafer (Findikli Gofret)</t>
+        </is>
+      </c>
+      <c r="M54" s="90" t="inlineStr">
+        <is>
+          <t>Assigned Label
+Cloze: 'Hazelnut wafer has been given ___ as label' → not recommended (tavsiye edilemez)</t>
         </is>
       </c>
       <c r="N54" s="85" t="inlineStr">
@@ -6430,25 +6460,25 @@
       </c>
       <c r="C3" s="82" t="inlineStr">
         <is>
-          <t>Task 1
+          <t>Blank 1
 Circle 4 misclassified</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
-          <t>Task 2
+          <t>Blank 2
 Better threshold position</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>Exercise 3
+          <t>Blank 3
 Pia correct?</t>
         </is>
       </c>
       <c r="F3" s="82" t="inlineStr">
         <is>
-          <t>Task 4
+          <t>Blank 4
 Best energy threshold</t>
         </is>
       </c>
@@ -6476,13 +6506,13 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -7015,13 +7045,13 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -7293,20 +7323,19 @@
       <c r="G51" s="85" t="n"/>
       <c r="H51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
-      <c r="H53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="86" t="n"/>
+      <c r="H53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -7315,24 +7344,28 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>Task 1: Circles all 4 incorrectly classified food cards at Leo's threshold</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>Task 2: Places threshold between two adjacent distinct fat values; written justification present</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>Exercise 3: Explains why equal-valued items cannot be split (Pia is correct; equal values cannot be separated)</t>
-        </is>
-      </c>
-      <c r="F54" s="85" t="inlineStr">
-        <is>
-          <t>Task 4: Sorts cards, fills table, writes best energy threshold in final blank</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Circle 4 misclassified
+Circles all 4 incorrectly classified food cards at Leo's threshold</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>Better threshold position
+Places threshold between two adjacent distinct fat values; written justification present</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Pia correct?
+Explains why equal-valued items cannot be split (Pia is correct; equal values cannot be separated)</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>Best energy threshold
+Sorts cards, fills table, writes best energy threshold in final blank</t>
         </is>
       </c>
       <c r="G54" s="85" t="inlineStr">
@@ -7463,43 +7496,43 @@
       </c>
       <c r="C3" s="82" t="inlineStr">
         <is>
-          <t>Block 1
+          <t>Blank 1
 Variable + threshold</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
-          <t>Block 1
+          <t>Blank 2
 Count consistency</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>Block 2
+          <t>Blank 3
 Variable + threshold</t>
         </is>
       </c>
       <c r="F3" s="82" t="inlineStr">
         <is>
-          <t>Block 2
+          <t>Blank 4
 Count consistency</t>
         </is>
       </c>
       <c r="G3" s="82" t="inlineStr">
         <is>
-          <t>Block 3
+          <t>Blank 5
 Variable + threshold</t>
         </is>
       </c>
       <c r="H3" s="82" t="inlineStr">
         <is>
-          <t>Block 3
+          <t>Blank 6
 Count consistency</t>
         </is>
       </c>
       <c r="I3" s="82" t="inlineStr">
         <is>
-          <t>Final blank
+          <t>Blank 7
 Chosen threshold</t>
         </is>
       </c>
@@ -7527,16 +7560,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -8156,16 +8189,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -8482,23 +8515,22 @@
       <c r="J51" s="85" t="n"/>
       <c r="K51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
-      <c r="H53" s="84" t="n"/>
-      <c r="I53" s="84" t="n"/>
-      <c r="J53" s="84" t="n"/>
-      <c r="K53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="86" t="n"/>
+      <c r="H53" s="86" t="n"/>
+      <c r="I53" s="86" t="n"/>
+      <c r="J53" s="86" t="n"/>
+      <c r="K53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -8507,39 +8539,46 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>Block 1: Names a valid dataset variable and fills in threshold value(s)</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>Block 1: Recommended + not-recommended counts sum correctly to total number of cards</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>Block 2: Names a different valid variable and fills in threshold value(s)</t>
-        </is>
-      </c>
-      <c r="F54" s="85" t="inlineStr">
-        <is>
-          <t>Block 2: Counts sum correctly</t>
-        </is>
-      </c>
-      <c r="G54" s="85" t="inlineStr">
-        <is>
-          <t>Block 3: Names a third valid variable and fills in threshold value(s)</t>
-        </is>
-      </c>
-      <c r="H54" s="85" t="inlineStr">
-        <is>
-          <t>Block 3: Counts sum correctly</t>
-        </is>
-      </c>
-      <c r="I54" s="85" t="inlineStr">
-        <is>
-          <t>Final line: states which variable and threshold they selected and records it</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Variable + threshold
+Names a valid dataset variable and fills in threshold value(s)</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>Count consistency
+Recommended + not-recommended counts sum correctly to total number of cards</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Variable + threshold
+Names a different valid variable and fills in threshold value(s)</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>Count consistency
+Counts sum correctly</t>
+        </is>
+      </c>
+      <c r="G54" s="90" t="inlineStr">
+        <is>
+          <t>Variable + threshold
+Names a third valid variable and fills in threshold value(s)</t>
+        </is>
+      </c>
+      <c r="H54" s="90" t="inlineStr">
+        <is>
+          <t>Count consistency
+Counts sum correctly</t>
+        </is>
+      </c>
+      <c r="I54" s="90" t="inlineStr">
+        <is>
+          <t>Chosen threshold
+Final line: states which variable and threshold they selected and records it</t>
         </is>
       </c>
       <c r="J54" s="85" t="inlineStr">
@@ -8670,43 +8709,43 @@
       </c>
       <c r="C3" s="82" t="inlineStr">
         <is>
-          <t>Root node
+          <t>Blank 1
 Variable</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
-          <t>Branch labels
+          <t>Blank 2
 &lt;= and &gt;</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>Left leaf
+          <t>Blank 3
 Classification</t>
         </is>
       </c>
       <c r="F3" s="82" t="inlineStr">
         <is>
-          <t>Left leaf
+          <t>Blank 4
 Counts</t>
         </is>
       </c>
       <c r="G3" s="82" t="inlineStr">
         <is>
-          <t>Right leaf
+          <t>Blank 5
 Classification</t>
         </is>
       </c>
       <c r="H3" s="82" t="inlineStr">
         <is>
-          <t>Right leaf
+          <t>Blank 6
 Counts</t>
         </is>
       </c>
       <c r="I3" s="82" t="inlineStr">
         <is>
-          <t>2nd level node
+          <t>Blank 7
 Variable (if present)</t>
         </is>
       </c>
@@ -8734,16 +8773,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -9363,16 +9402,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -9689,23 +9728,22 @@
       <c r="J51" s="85" t="n"/>
       <c r="K51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
-      <c r="H53" s="84" t="n"/>
-      <c r="I53" s="84" t="n"/>
-      <c r="J53" s="84" t="n"/>
-      <c r="K53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="86" t="n"/>
+      <c r="H53" s="86" t="n"/>
+      <c r="I53" s="86" t="n"/>
+      <c r="J53" s="86" t="n"/>
+      <c r="K53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -9714,39 +9752,46 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>Root node blank: names a variable for the first split</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>Branch labels: writes &lt;= and &gt; with threshold values on both branches</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>Left leaf: correct classification label (recommended / not recommended)</t>
-        </is>
-      </c>
-      <c r="F54" s="85" t="inlineStr">
-        <is>
-          <t>Left leaf: correct counts in brackets [recommended] [not-recommended]</t>
-        </is>
-      </c>
-      <c r="G54" s="85" t="inlineStr">
-        <is>
-          <t>Right leaf: correct classification label</t>
-        </is>
-      </c>
-      <c r="H54" s="85" t="inlineStr">
-        <is>
-          <t>Right leaf: correct counts in brackets</t>
-        </is>
-      </c>
-      <c r="I54" s="85" t="inlineStr">
-        <is>
-          <t>Second-level node: names a valid variable for further split (score if present)</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Variable
+Root node blank: names a variable for the first split</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>&lt;= and &gt;
+Branch labels: writes &lt;= and &gt; with threshold values on both branches</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Classification
+Left leaf: correct classification label (recommended / not recommended)</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>Counts
+Left leaf: correct counts in brackets [recommended] [not-recommended]</t>
+        </is>
+      </c>
+      <c r="G54" s="90" t="inlineStr">
+        <is>
+          <t>Classification
+Right leaf: correct classification label</t>
+        </is>
+      </c>
+      <c r="H54" s="90" t="inlineStr">
+        <is>
+          <t>Counts
+Right leaf: correct counts in brackets</t>
+        </is>
+      </c>
+      <c r="I54" s="90" t="inlineStr">
+        <is>
+          <t>Variable (if present)
+Second-level node: names a valid variable for further split (score if present)</t>
         </is>
       </c>
       <c r="J54" s="85" t="inlineStr">
@@ -9877,43 +9922,43 @@
       </c>
       <c r="C3" s="82" t="inlineStr">
         <is>
-          <t>Page 1
+          <t>Blank 1
 Path A match</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
-          <t>Page 1
+          <t>Blank 2
 Path B match</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>Page 1
+          <t>Blank 3
 Path C match</t>
         </is>
       </c>
       <c r="F3" s="82" t="inlineStr">
         <is>
-          <t>Page 2
+          <t>Blank 4
 Path count</t>
         </is>
       </c>
       <c r="G3" s="82" t="inlineStr">
         <is>
-          <t>Page 2
+          <t>Blank 5
 Rule 1</t>
         </is>
       </c>
       <c r="H3" s="82" t="inlineStr">
         <is>
-          <t>Page 2
+          <t>Blank 6
 Rule 2</t>
         </is>
       </c>
       <c r="I3" s="82" t="inlineStr">
         <is>
-          <t>Page 2
+          <t>Blank 7
 Rules 3-6</t>
         </is>
       </c>
@@ -9941,16 +9986,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -10570,16 +10615,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -10896,23 +10941,22 @@
       <c r="J51" s="85" t="n"/>
       <c r="K51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
-      <c r="H53" s="84" t="n"/>
-      <c r="I53" s="84" t="n"/>
-      <c r="J53" s="84" t="n"/>
-      <c r="K53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="86" t="n"/>
+      <c r="H53" s="86" t="n"/>
+      <c r="I53" s="86" t="n"/>
+      <c r="J53" s="86" t="n"/>
+      <c r="K53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -10921,39 +10965,46 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>Page 1 matching: assigns correct rule to Path A (energy &lt; 180 kcal -&gt; recommended)</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>Page 1 matching: assigns correct rule to Path B (energy &gt;= 180 AND protein &lt; 7.7 -&gt; not recommended)</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>Page 1 matching: assigns correct rule to Path C (energy &gt;= 180 AND protein &gt;= 7.7 -&gt; recommended)</t>
-        </is>
-      </c>
-      <c r="F54" s="85" t="inlineStr">
-        <is>
-          <t>Page 2 blank: 'My tree contains ___ paths' — states correct number of paths</t>
-        </is>
-      </c>
-      <c r="G54" s="85" t="inlineStr">
-        <is>
-          <t>Page 2 Rule 1: writes a complete if-then rule logically consistent with their WS6 tree</t>
-        </is>
-      </c>
-      <c r="H54" s="85" t="inlineStr">
-        <is>
-          <t>Page 2 Rule 2: second rule consistent with tree</t>
-        </is>
-      </c>
-      <c r="I54" s="85" t="inlineStr">
-        <is>
-          <t>Page 2 Rules 3-6: additional rules present and consistent (score if all paths covered)</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Path A match
+Page 1 matching: assigns correct rule to Path A (energy &lt; 180 kcal -&gt; recommended)</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>Path B match
+Page 1 matching: assigns correct rule to Path B (energy &gt;= 180 AND protein &lt; 7.7 -&gt; not recommended)</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Path C match
+Page 1 matching: assigns correct rule to Path C (energy &gt;= 180 AND protein &gt;= 7.7 -&gt; recommended)</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>Path count
+Page 2 blank: 'My tree contains ___ paths' — states correct number of paths</t>
+        </is>
+      </c>
+      <c r="G54" s="90" t="inlineStr">
+        <is>
+          <t>Rule 1
+Page 2 Rule 1: writes a complete if-then rule logically consistent with their WS6 tree</t>
+        </is>
+      </c>
+      <c r="H54" s="90" t="inlineStr">
+        <is>
+          <t>Rule 2
+Page 2 Rule 2: second rule consistent with tree</t>
+        </is>
+      </c>
+      <c r="I54" s="90" t="inlineStr">
+        <is>
+          <t>Rules 3-6
+Page 2 Rules 3-6: additional rules present and consistent (score if all paths covered)</t>
         </is>
       </c>
       <c r="J54" s="85" t="inlineStr">
@@ -11060,19 +11111,19 @@
       </c>
       <c r="C3" s="82" t="inlineStr">
         <is>
-          <t>Table
+          <t>Blank 1
 Misclassification counts</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
-          <t>Final blank
+          <t>Blank 2
 Optimum threshold</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>Reasoning
+          <t>Blank 3
 Why optimum</t>
         </is>
       </c>
@@ -11100,12 +11151,12 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -11609,12 +11660,12 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -11871,19 +11922,18 @@
       <c r="F51" s="85" t="n"/>
       <c r="G51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -11892,19 +11942,22 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>Table: correctly counts misclassifications for each of the 7 candidate thresholds</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>Final blank: 'The optimum threshold is: ___' — selects threshold with fewest errors</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>Written justification: explains why this threshold minimizes error (score if present)</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Misclassification counts
+Table: correctly counts misclassifications for each of the 7 candidate thresholds</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>Optimum threshold
+Final blank: 'The optimum threshold is: ___' — selects threshold with fewest errors</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Why optimum
+Written justification: explains why this threshold minimizes error (score if present)</t>
         </is>
       </c>
       <c r="F54" s="85" t="inlineStr">
@@ -12035,43 +12088,43 @@
       </c>
       <c r="C3" s="82" t="inlineStr">
         <is>
-          <t>Q4
+          <t>Blank 1
 Can explain DT</t>
         </is>
       </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
-          <t>Q8a
+          <t>Blank 2
 Classify strawberry</t>
         </is>
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>Q8b
+          <t>Blank 3
 Decision rule</t>
         </is>
       </c>
       <c r="F3" s="82" t="inlineStr">
         <is>
-          <t>Q9
+          <t>Blank 4
 What is data</t>
         </is>
       </c>
       <c r="G3" s="82" t="inlineStr">
         <is>
-          <t>Q10
+          <t>Blank 5
 DT capabilities</t>
         </is>
       </c>
       <c r="H3" s="82" t="inlineStr">
         <is>
-          <t>Q11
+          <t>Blank 6
 Step ordering</t>
         </is>
       </c>
       <c r="I3" s="82" t="inlineStr">
         <is>
-          <t>Q12
+          <t>Blank 7
 Why is DT AI</t>
         </is>
       </c>
@@ -12099,16 +12152,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="n"/>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="51">
       <c r="A6" s="85" t="inlineStr">
@@ -12728,16 +12781,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n"/>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="51">
       <c r="A37" s="85" t="inlineStr">
@@ -13054,23 +13107,22 @@
       <c r="J51" s="85" t="n"/>
       <c r="K51" s="85" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="84" t="inlineStr">
         <is>
           <t>Dropdown values: Acquire | Deepen | Create | ? (unscorable/blank)</t>
         </is>
       </c>
-      <c r="B53" s="84" t="n"/>
-      <c r="C53" s="84" t="n"/>
-      <c r="D53" s="84" t="n"/>
-      <c r="E53" s="84" t="n"/>
-      <c r="F53" s="84" t="n"/>
-      <c r="G53" s="84" t="n"/>
-      <c r="H53" s="84" t="n"/>
-      <c r="I53" s="84" t="n"/>
-      <c r="J53" s="84" t="n"/>
-      <c r="K53" s="84" t="n"/>
+      <c r="B53" s="86" t="n"/>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="86" t="n"/>
+      <c r="E53" s="86" t="n"/>
+      <c r="F53" s="86" t="n"/>
+      <c r="G53" s="86" t="n"/>
+      <c r="H53" s="86" t="n"/>
+      <c r="I53" s="86" t="n"/>
+      <c r="J53" s="86" t="n"/>
+      <c r="K53" s="87" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1" s="51">
       <c r="A54" s="85" t="inlineStr">
@@ -13079,39 +13131,46 @@
         </is>
       </c>
       <c r="B54" s="85" t="n"/>
-      <c r="C54" s="85" t="inlineStr">
-        <is>
-          <t>Q4 (yes/no): Can you explain how a decision tree works? Score as Acquire if 'Yes'</t>
-        </is>
-      </c>
-      <c r="D54" s="85" t="inlineStr">
-        <is>
-          <t>Q8a: Uses the given decision tree to classify strawberries correctly</t>
-        </is>
-      </c>
-      <c r="E54" s="85" t="inlineStr">
-        <is>
-          <t>Q8b: Writes correct decision rule for strawberry classification (blank: ___ because ___)</t>
-        </is>
-      </c>
-      <c r="F54" s="85" t="inlineStr">
-        <is>
-          <t>Q9: Open-ended (6 lines) — explains what data is and why we need it</t>
-        </is>
-      </c>
-      <c r="G54" s="85" t="inlineStr">
-        <is>
-          <t>Q10: Multi-select T/F table — marks correct statements about what DTs can do</t>
-        </is>
-      </c>
-      <c r="H54" s="85" t="inlineStr">
-        <is>
-          <t>Q11: Orders the 4 steps for building a decision rule correctly (1-4)</t>
-        </is>
-      </c>
-      <c r="I54" s="85" t="inlineStr">
-        <is>
-          <t>Q12: Multi-select T/F table — marks correct reasons why a DT is considered AI</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Can explain DT
+Q4 (yes/no): Can you explain how a decision tree works? Score as Acquire if 'Yes'</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>Classify strawberry
+Uses the given decision tree to classify strawberries correctly</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>Decision rule
+Writes correct decision rule for strawberry classification (blank: ___ because ___)</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>What is data
+Open-ended (6 lines) — explains what data is and why we need it</t>
+        </is>
+      </c>
+      <c r="G54" s="90" t="inlineStr">
+        <is>
+          <t>DT capabilities
+Multi-select T/F table — marks correct statements about what DTs can do</t>
+        </is>
+      </c>
+      <c r="H54" s="90" t="inlineStr">
+        <is>
+          <t>Step ordering
+Orders the 4 steps for building a decision rule correctly (1-4)</t>
+        </is>
+      </c>
+      <c r="I54" s="90" t="inlineStr">
+        <is>
+          <t>Why is DT AI
+Multi-select T/F table — marks correct reasons why a DT is considered AI</t>
         </is>
       </c>
       <c r="J54" s="85" t="inlineStr">

</xml_diff>

<commit_message>
Row 3: titles only; Row 54: descriptions only, all sheets
</commit_message>
<xml_diff>
--- a/AI_CFT_Labeling.xlsx
+++ b/AI_CFT_Labeling.xlsx
@@ -434,7 +434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -685,6 +685,9 @@
     <xf numFmtId="0" fontId="25" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1768,37 +1771,33 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
-      <c r="L5" s="84" t="n"/>
-      <c r="M5" s="84" t="n"/>
-      <c r="N5" s="84" t="n"/>
-      <c r="O5" s="84" t="n"/>
-      <c r="P5" s="84" t="n"/>
-      <c r="Q5" s="84" t="n"/>
-      <c r="R5" s="84" t="n"/>
-      <c r="S5" s="84" t="n"/>
-      <c r="T5" s="84" t="n"/>
-      <c r="U5" s="84" t="n"/>
-      <c r="V5" s="84" t="n"/>
-      <c r="W5" s="84" t="n"/>
-      <c r="X5" s="84" t="n"/>
-      <c r="Y5" s="84" t="n"/>
-      <c r="Z5" s="84" t="n"/>
-      <c r="AA5" s="84" t="n"/>
-      <c r="AB5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="86" t="n"/>
+      <c r="L5" s="86" t="n"/>
+      <c r="M5" s="86" t="n"/>
+      <c r="N5" s="86" t="n"/>
+      <c r="O5" s="86" t="n"/>
+      <c r="P5" s="86" t="n"/>
+      <c r="Q5" s="86" t="n"/>
+      <c r="R5" s="86" t="n"/>
+      <c r="S5" s="86" t="n"/>
+      <c r="T5" s="86" t="n"/>
+      <c r="U5" s="86" t="n"/>
+      <c r="V5" s="86" t="n"/>
+      <c r="W5" s="86" t="n"/>
+      <c r="X5" s="86" t="n"/>
+      <c r="Y5" s="86" t="n"/>
+      <c r="Z5" s="86" t="n"/>
+      <c r="AA5" s="86" t="n"/>
+      <c r="AB5" s="87" t="n"/>
       <c r="AC5" s="84" t="n"/>
       <c r="AD5" s="84" t="n"/>
       <c r="AE5" s="84" t="n"/>
@@ -3065,37 +3064,33 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
-      <c r="L36" s="84" t="n"/>
-      <c r="M36" s="84" t="n"/>
-      <c r="N36" s="84" t="n"/>
-      <c r="O36" s="84" t="n"/>
-      <c r="P36" s="84" t="n"/>
-      <c r="Q36" s="84" t="n"/>
-      <c r="R36" s="84" t="n"/>
-      <c r="S36" s="84" t="n"/>
-      <c r="T36" s="84" t="n"/>
-      <c r="U36" s="84" t="n"/>
-      <c r="V36" s="84" t="n"/>
-      <c r="W36" s="84" t="n"/>
-      <c r="X36" s="84" t="n"/>
-      <c r="Y36" s="84" t="n"/>
-      <c r="Z36" s="84" t="n"/>
-      <c r="AA36" s="84" t="n"/>
-      <c r="AB36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="86" t="n"/>
+      <c r="L36" s="86" t="n"/>
+      <c r="M36" s="86" t="n"/>
+      <c r="N36" s="86" t="n"/>
+      <c r="O36" s="86" t="n"/>
+      <c r="P36" s="86" t="n"/>
+      <c r="Q36" s="86" t="n"/>
+      <c r="R36" s="86" t="n"/>
+      <c r="S36" s="86" t="n"/>
+      <c r="T36" s="86" t="n"/>
+      <c r="U36" s="86" t="n"/>
+      <c r="V36" s="86" t="n"/>
+      <c r="W36" s="86" t="n"/>
+      <c r="X36" s="86" t="n"/>
+      <c r="Y36" s="86" t="n"/>
+      <c r="Z36" s="86" t="n"/>
+      <c r="AA36" s="86" t="n"/>
+      <c r="AB36" s="87" t="n"/>
       <c r="AC36" s="84" t="n"/>
       <c r="AD36" s="84" t="n"/>
       <c r="AE36" s="84" t="n"/>
@@ -3757,176 +3752,147 @@
     <row r="54" ht="60" customHeight="1" s="51">
       <c r="C54" s="93" t="inlineStr">
         <is>
-          <t>A1 – Prior belief
-Which variables do you predict will determine recommendability? (intuition, no analysis yet)</t>
+          <t>Which variables do you predict will determine recommendability? (intuition, no analysis yet)</t>
         </is>
       </c>
       <c r="D54" s="93" t="inlineStr">
         <is>
-          <t>A2 – Data-based exploration
-Which variables actually influence recommendability based on data? (with graph evidence)</t>
+          <t>Which variables actually influence recommendability based on data? (with graph evidence)</t>
         </is>
       </c>
       <c r="E54" s="93" t="inlineStr">
         <is>
-          <t>A3 – Meaningful difference
-Did you find a variable showing meaningful difference between groups? Explain with data.</t>
+          <t>Did you find a variable showing meaningful difference between groups? Explain with data.</t>
         </is>
       </c>
       <c r="F54" s="93" t="inlineStr">
         <is>
-          <t>A4 – First variable justification
-Which variable would you use first in a prediction model? Justify using data evidence.</t>
+          <t>Which variable would you use first in a prediction model? Justify using data evidence.</t>
         </is>
       </c>
       <c r="G54" s="93" t="inlineStr">
         <is>
-          <t>B1 – Tree 1 build + EMIT
-Build single-level tree with variable 1; record EMIT accuracy result</t>
+          <t>Build single-level tree with variable 1; record EMIT accuracy result</t>
         </is>
       </c>
       <c r="H54" s="93" t="inlineStr">
         <is>
-          <t>B2 – Tree 2 build + EMIT
-Build single-level tree with variable 2; record EMIT accuracy result</t>
+          <t>Build single-level tree with variable 2; record EMIT accuracy result</t>
         </is>
       </c>
       <c r="I54" s="93" t="inlineStr">
         <is>
-          <t>B3 – Tree 3 build + EMIT
-Build single-level tree with variable 3; record EMIT accuracy result</t>
+          <t>Build single-level tree with variable 3; record EMIT accuracy result</t>
         </is>
       </c>
       <c r="J54" s="93" t="inlineStr">
         <is>
-          <t>B4 – Best tree + criteria
-Which variable gave best result? What criteria used to judge?</t>
+          <t>Which variable gave best result? What criteria used to judge?</t>
         </is>
       </c>
       <c r="K54" s="93" t="inlineStr">
         <is>
-          <t>C1 – Threshold optimization
-Try different thresholds for best variable; save best result with EMIT</t>
+          <t>Try different thresholds for best variable; save best result with EMIT</t>
         </is>
       </c>
       <c r="L54" s="93" t="inlineStr">
         <is>
-          <t>C2 – Threshold effect
-How does changing the threshold value affect decision tree performance?</t>
+          <t>How does changing the threshold value affect decision tree performance?</t>
         </is>
       </c>
       <c r="M54" s="93" t="inlineStr">
         <is>
-          <t>C3 – Best threshold + reasoning
-Which threshold best separates the groups? How did you decide?</t>
+          <t>Which threshold best separates the groups? How did you decide?</t>
         </is>
       </c>
       <c r="N54" s="93" t="inlineStr">
         <is>
-          <t>D1 – Two-level tree build + EMIT
-Add second variable to create a two-level tree; save result with EMIT</t>
+          <t>Add second variable to create a two-level tree; save result with EMIT</t>
         </is>
       </c>
       <c r="O54" s="93" t="inlineStr">
         <is>
-          <t>D2 – Second level effect
-Did the second level improve classification? How and in what ways?</t>
+          <t>Did the second level improve classification? How and in what ways?</t>
         </is>
       </c>
       <c r="P54" s="93" t="inlineStr">
         <is>
-          <t>D3 – Best variable combination
-Which variable combination produced the best result?</t>
+          <t>Which variable combination produced the best result?</t>
         </is>
       </c>
       <c r="Q54" s="93" t="inlineStr">
         <is>
-          <t>D4 – Stopping criterion
-How did you decide you had reached your best decision tree?</t>
+          <t>How did you decide you had reached your best decision tree?</t>
         </is>
       </c>
       <c r="R54" s="93" t="inlineStr">
         <is>
-          <t>E – Sensitivity value
-Fill in Sensitivity (Duyarlılık) value from EMIT for best tree</t>
+          <t>Fill in Sensitivity (Duyarlılık) value from EMIT for best tree</t>
         </is>
       </c>
       <c r="S54" s="93" t="inlineStr">
         <is>
-          <t>E – MCR value
-Fill in Misclassification Rate (MCR) value from EMIT for best tree</t>
+          <t>Fill in Misclassification Rate (MCR) value from EMIT for best tree</t>
         </is>
       </c>
       <c r="T54" s="93" t="inlineStr">
         <is>
-          <t>E – True Positives
-Count of True Positives (TP) from confusion matrix</t>
+          <t>Count of True Positives (TP) from confusion matrix</t>
         </is>
       </c>
       <c r="U54" s="93" t="inlineStr">
         <is>
-          <t>E – False Positives
-Count of False Positives (FP) from confusion matrix</t>
+          <t>Count of False Positives (FP) from confusion matrix</t>
         </is>
       </c>
       <c r="V54" s="93" t="inlineStr">
         <is>
-          <t>E – True Negatives
-Count of True Negatives (TN) from confusion matrix</t>
+          <t>Count of True Negatives (TN) from confusion matrix</t>
         </is>
       </c>
       <c r="W54" s="93" t="inlineStr">
         <is>
-          <t>E – False Negatives
-Count of False Negatives (FN) from confusion matrix</t>
+          <t>Count of False Negatives (FN) from confusion matrix</t>
         </is>
       </c>
       <c r="X54" s="93" t="inlineStr">
         <is>
-          <t>E1 – Metric interpretation
-Which metric matters most for this model's purpose: sensitivity, MCR, or other? Why?</t>
+          <t>Which metric matters most for this model's purpose: sensitivity, MCR, or other? Why?</t>
         </is>
       </c>
       <c r="Y54" s="93" t="inlineStr">
         <is>
-          <t>E2 – Error type analysis
-Did model make more false positives or false negatives?</t>
+          <t>Did model make more false positives or false negatives?</t>
         </is>
       </c>
       <c r="Z54" s="93" t="inlineStr">
         <is>
-          <t>E3 – Good-enough criterion
-How would software / you decide when a tree is good enough?</t>
+          <t>How would software / you decide when a tree is good enough?</t>
         </is>
       </c>
       <c r="AA54" s="93" t="inlineStr">
         <is>
-          <t>E4 – Perfect classification
-Do you think decision trees can ever classify perfectly? Reasoned answer.</t>
+          <t>Do you think decision trees can ever classify perfectly? Reasoned answer.</t>
         </is>
       </c>
       <c r="AB54" s="93" t="inlineStr">
         <is>
-          <t>F1 – Test set application
-Apply best tree to test dataset; evaluate with EMIT; record result</t>
+          <t>Apply best tree to test dataset; evaluate with EMIT; record result</t>
         </is>
       </c>
       <c r="AC54" s="93" t="inlineStr">
         <is>
-          <t>F2 – Train vs test comparison
-Compare test vs. training performance and explain any difference</t>
+          <t>Compare test vs. training performance and explain any difference</t>
         </is>
       </c>
       <c r="AD54" s="93" t="inlineStr">
         <is>
-          <t>G1 – What the model learned
-What did the decision tree model 'learn' from the training data?</t>
+          <t>What did the decision tree model 'learn' from the training data?</t>
         </is>
       </c>
       <c r="AE54" s="93" t="inlineStr">
         <is>
-          <t>G2 – Personal reflection
-What did you personally learn while building decision trees?</t>
+          <t>What did you personally learn while building decision trees?</t>
         </is>
       </c>
     </row>
@@ -5334,75 +5300,60 @@
       <c r="B54" s="85" t="n"/>
       <c r="C54" s="90" t="inlineStr">
         <is>
-          <t>Target Label
-Diagram arrow pointing to food card name → 'label' (etiket)</t>
+          <t>Diagram arrow pointing to food card name → 'label' (etiket)</t>
         </is>
       </c>
       <c r="D54" s="90" t="inlineStr">
         <is>
-          <t>Data Object
-Diagram arrow pointing to 'Findikli Gofret' card → 'object' (nesne)</t>
+          <t>Diagram arrow pointing to 'Findikli Gofret' card → 'object' (nesne)</t>
         </is>
       </c>
       <c r="E54" s="90" t="inlineStr">
         <is>
-          <t>Feature Name
-Diagram arrow pointing to left column of card → 'feature / variable / characteristic'</t>
+          <t>Diagram arrow pointing to left column of card → 'feature / variable / characteristic'</t>
         </is>
       </c>
       <c r="F54" s="90" t="inlineStr">
         <is>
-          <t>Feature Value
-Diagram arrow pointing to a numeric cell → 'value of the feature / characteristic'</t>
+          <t>Diagram arrow pointing to a numeric cell → 'value of the feature / characteristic'</t>
         </is>
       </c>
       <c r="G54" s="90" t="inlineStr">
         <is>
-          <t>Data Instance
-Cloze: 'Individual foods are called ___' → object (nesne)</t>
+          <t>Cloze: 'Individual foods are called ___' → object (nesne)</t>
         </is>
       </c>
       <c r="H54" s="90" t="inlineStr">
         <is>
-          <t>Specific Object
-Cloze: 'Hazelnut wafer is a ___' → object (nesne)</t>
+          <t>Cloze: 'Hazelnut wafer is a ___' → object (nesne)</t>
         </is>
       </c>
       <c r="I54" s="90" t="inlineStr">
         <is>
-          <t>Feature Variable
-Cloze: left-column names are called '___ / characteristic / variable'</t>
+          <t>Cloze: left-column names are called '___ / characteristic / variable'</t>
         </is>
       </c>
       <c r="J54" s="90" t="inlineStr">
         <is>
-          <t>Feature Count
-Cloze: 'How many features? ___' → 7 (yedi / seven)</t>
+          <t>Cloze: 'How many features? ___' → 7 (yedi / seven)</t>
         </is>
       </c>
       <c r="K54" s="90" t="inlineStr">
         <is>
-          <t>Feature List
-Cloze: student writes all feature names: Energy, Fat, Saturated Fat, Carbohydrates, Sugar, Protein, Salt</t>
+          <t>Cloze: student writes all feature names: Energy, Fat, Saturated Fat, Carbohydrates, Sugar, Protein, Salt</t>
         </is>
       </c>
       <c r="L54" s="90" t="inlineStr">
         <is>
-          <t>Instance Name
-Cloze: 'For example ___ contains 31.9g fat' → Hazelnut Wafer (Findikli Gofret)</t>
+          <t>Cloze: 'For example ___ contains 31.9g fat' → Hazelnut Wafer (Findikli Gofret)</t>
         </is>
       </c>
       <c r="M54" s="90" t="inlineStr">
         <is>
-          <t>Assigned Label
-Cloze: 'Hazelnut wafer has been given ___ as label' → not recommended (tavsiye edilemez)</t>
-        </is>
-      </c>
-      <c r="N54" s="85" t="inlineStr">
-        <is>
-          <t>Overall AI-CFT level for WS1 as a whole</t>
-        </is>
-      </c>
+          <t>Cloze: 'Hazelnut wafer has been given ___ as label' → not recommended (tavsiye edilemez)</t>
+        </is>
+      </c>
+      <c r="N54" s="85" t="n"/>
       <c r="O54" s="85" t="inlineStr">
         <is>
           <t>Free notes: edge cases, illegible answers, etc.</t>
@@ -6632,42 +6583,42 @@
         </is>
       </c>
       <c r="B54" s="25" t="n"/>
-      <c r="C54" s="35" t="inlineStr">
+      <c r="C54" s="94" t="inlineStr">
         <is>
           <t>Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
         </is>
       </c>
-      <c r="D54" s="35" t="inlineStr">
+      <c r="D54" s="94" t="inlineStr">
         <is>
           <t>Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "23.0 &gt; 8.0").</t>
         </is>
       </c>
-      <c r="E54" s="35" t="inlineStr">
+      <c r="E54" s="94" t="inlineStr">
         <is>
           <t>Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilebilir").</t>
         </is>
       </c>
-      <c r="F54" s="35" t="inlineStr">
+      <c r="F54" s="94" t="inlineStr">
         <is>
           <t>Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "8.0 &gt; 0.2").</t>
         </is>
       </c>
-      <c r="G54" s="35" t="inlineStr">
+      <c r="G54" s="94" t="inlineStr">
         <is>
           <t>Applying the established decision rule to predict and assign a target class label to a specific data object (e.g., "tavsiye edilemez").</t>
         </is>
       </c>
-      <c r="H54" s="35" t="inlineStr">
+      <c r="H54" s="94" t="inlineStr">
         <is>
           <t>Justifying the classification outcome by mathematically comparing the object's feature value to the threshold (e.g., "14.0 &gt; 8.0").</t>
         </is>
       </c>
-      <c r="I54" s="36" t="inlineStr">
+      <c r="I54" s="93" t="inlineStr">
         <is>
           <t>Establishing the mathematical boundary expression (≤) for a split node based on the data distribution of the feature (e.g., ≤ 71 kcal).</t>
         </is>
       </c>
-      <c r="J54" s="36" t="inlineStr">
+      <c r="J54" s="93" t="inlineStr">
         <is>
           <t>Establishing the corresponding inverse mathematical expression (&gt;) for a split node to partition the remaining instances in the dataset (e.g., &gt; 71 kcal).</t>
         </is>
@@ -6842,17 +6793,13 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="87" t="n"/>
       <c r="I5" s="84" t="n"/>
       <c r="J5" s="84" t="n"/>
     </row>
@@ -7449,17 +7396,13 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="87" t="n"/>
       <c r="I36" s="84" t="n"/>
       <c r="J36" s="84" t="n"/>
     </row>
@@ -7773,38 +7716,32 @@
     <row r="54" ht="60" customHeight="1" s="51">
       <c r="C54" s="93" t="inlineStr">
         <is>
-          <t>Circle 4 misclassified
-Identify which 4 food cards are incorrectly classified at Leo's threshold</t>
+          <t>Identify which 4 food cards are incorrectly classified at Leo's threshold</t>
         </is>
       </c>
       <c r="D54" s="93" t="inlineStr">
         <is>
-          <t>Better threshold position
-Mark a better threshold line between two adjacent foods on the sorted card row</t>
+          <t>Mark a better threshold line between two adjacent foods on the sorted card row</t>
         </is>
       </c>
       <c r="E54" s="93" t="inlineStr">
         <is>
-          <t>Threshold justification
-Written explanation of why chosen threshold is better than Leo's</t>
+          <t>Written explanation of why chosen threshold is better than Leo's</t>
         </is>
       </c>
       <c r="F54" s="93" t="inlineStr">
         <is>
-          <t>Pia correct?
-Explanation of why Leo's exact pencil placement cannot be a valid threshold (equal values cannot be split)</t>
+          <t>Explanation of why Leo's exact pencil placement cannot be a valid threshold (equal values cannot be split)</t>
         </is>
       </c>
       <c r="G54" s="93" t="inlineStr">
         <is>
-          <t>Sorted cards annotation
-Sort and annotate energy cards with the best threshold line drawn</t>
+          <t>Sort and annotate energy cards with the best threshold line drawn</t>
         </is>
       </c>
       <c r="H54" s="93" t="inlineStr">
         <is>
-          <t>Best energy threshold value
-Fill in: 'Best threshold value for energy variable: ___' (numerical value)</t>
+          <t>Fill in: 'Best threshold value for energy variable: ___' (numerical value)</t>
         </is>
       </c>
     </row>
@@ -8247,20 +8184,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
       <c r="L5" s="84" t="n"/>
       <c r="M5" s="84" t="n"/>
       <c r="N5" s="84" t="n"/>
@@ -9514,20 +9447,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
       <c r="L36" s="84" t="n"/>
       <c r="M36" s="84" t="n"/>
       <c r="N36" s="84" t="n"/>
@@ -10190,170 +10119,142 @@
     <row r="54" ht="60" customHeight="1" s="51">
       <c r="C54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Variable name
-Name of first chosen variable for threshold exploration</t>
+          <t>Name of first chosen variable for threshold exploration</t>
         </is>
       </c>
       <c r="D54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Threshold ≤
-Left threshold value (≤ side) for variable 1</t>
+          <t>Left threshold value (≤ side) for variable 1</t>
         </is>
       </c>
       <c r="E54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Threshold &gt;
-Right threshold value (&gt; side) for variable 1</t>
+          <t>Right threshold value (&gt; side) for variable 1</t>
         </is>
       </c>
       <c r="F54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Rec count (left)
-Count of recommended foods in left branch (variable 1)</t>
+          <t>Count of recommended foods in left branch (variable 1)</t>
         </is>
       </c>
       <c r="G54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Not-rec count (left)
-Count of not-recommended foods in left branch (variable 1)</t>
+          <t>Count of not-recommended foods in left branch (variable 1)</t>
         </is>
       </c>
       <c r="H54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Rec count (right)
-Count of recommended foods in right branch (variable 1)</t>
+          <t>Count of recommended foods in right branch (variable 1)</t>
         </is>
       </c>
       <c r="I54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Not-rec count (right)
-Count of not-recommended foods in right branch (variable 1)</t>
+          <t>Count of not-recommended foods in right branch (variable 1)</t>
         </is>
       </c>
       <c r="J54" s="93" t="inlineStr">
         <is>
-          <t>Block 1 – Misclassification count
-Total misclassified foods for variable 1 threshold</t>
+          <t>Total misclassified foods for variable 1 threshold</t>
         </is>
       </c>
       <c r="K54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Variable name
-Name of second chosen variable</t>
+          <t>Name of second chosen variable</t>
         </is>
       </c>
       <c r="L54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Threshold ≤
-Left threshold value (≤ side) for variable 2</t>
+          <t>Left threshold value (≤ side) for variable 2</t>
         </is>
       </c>
       <c r="M54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Threshold &gt;
-Right threshold value (&gt; side) for variable 2</t>
+          <t>Right threshold value (&gt; side) for variable 2</t>
         </is>
       </c>
       <c r="N54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Rec count (left)
-Count of recommended foods in left branch (variable 2)</t>
+          <t>Count of recommended foods in left branch (variable 2)</t>
         </is>
       </c>
       <c r="O54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Not-rec count (left)
-Count of not-recommended foods in left branch (variable 2)</t>
+          <t>Count of not-recommended foods in left branch (variable 2)</t>
         </is>
       </c>
       <c r="P54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Rec count (right)
-Count of recommended foods in right branch (variable 2)</t>
+          <t>Count of recommended foods in right branch (variable 2)</t>
         </is>
       </c>
       <c r="Q54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Not-rec count (right)
-Count of not-recommended foods in right branch (variable 2)</t>
+          <t>Count of not-recommended foods in right branch (variable 2)</t>
         </is>
       </c>
       <c r="R54" s="93" t="inlineStr">
         <is>
-          <t>Block 2 – Misclassification count
-Total misclassified foods for variable 2 threshold</t>
+          <t>Total misclassified foods for variable 2 threshold</t>
         </is>
       </c>
       <c r="S54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Variable name
-Name of third chosen variable</t>
+          <t>Name of third chosen variable</t>
         </is>
       </c>
       <c r="T54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Threshold ≤
-Left threshold value (≤ side) for variable 3</t>
+          <t>Left threshold value (≤ side) for variable 3</t>
         </is>
       </c>
       <c r="U54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Threshold &gt;
-Right threshold value (&gt; side) for variable 3</t>
+          <t>Right threshold value (&gt; side) for variable 3</t>
         </is>
       </c>
       <c r="V54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Rec count (left)
-Count of recommended foods in left branch (variable 3)</t>
+          <t>Count of recommended foods in left branch (variable 3)</t>
         </is>
       </c>
       <c r="W54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Not-rec count (left)
-Count of not-recommended foods in left branch (variable 3)</t>
+          <t>Count of not-recommended foods in left branch (variable 3)</t>
         </is>
       </c>
       <c r="X54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Rec count (right)
-Count of recommended foods in right branch (variable 3)</t>
+          <t>Count of recommended foods in right branch (variable 3)</t>
         </is>
       </c>
       <c r="Y54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Not-rec count (right)
-Count of not-recommended foods in right branch (variable 3)</t>
+          <t>Count of not-recommended foods in right branch (variable 3)</t>
         </is>
       </c>
       <c r="Z54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Rec total
-Total recommended count across all branches (variable 3)</t>
+          <t>Total recommended count across all branches (variable 3)</t>
         </is>
       </c>
       <c r="AA54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Not-rec total
-Total not-recommended count across all branches (variable 3)</t>
+          <t>Total not-recommended count across all branches (variable 3)</t>
         </is>
       </c>
       <c r="AB54" s="93" t="inlineStr">
         <is>
-          <t>Block 3 – Misclassification count
-Total misclassified foods for variable 3 threshold</t>
+          <t>Total misclassified foods for variable 3 threshold</t>
         </is>
       </c>
       <c r="AC54" s="93" t="inlineStr">
         <is>
-          <t>Chosen variable
-Variable name selected as best for final threshold</t>
+          <t>Variable name selected as best for final threshold</t>
         </is>
       </c>
       <c r="AD54" s="93" t="inlineStr">
         <is>
-          <t>Selected threshold value
-'Which threshold do you choose for ___ variable?' — final numerical answer</t>
+          <t>'Which threshold do you choose for ___ variable?' — final numerical answer</t>
         </is>
       </c>
     </row>
@@ -10712,20 +10613,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
       <c r="L5" s="84" t="n"/>
       <c r="M5" s="84" t="n"/>
       <c r="N5" s="84" t="n"/>
@@ -11769,20 +11666,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
       <c r="L36" s="84" t="n"/>
       <c r="M36" s="84" t="n"/>
       <c r="N36" s="84" t="n"/>
@@ -12333,128 +12226,107 @@
     <row r="54" ht="60" customHeight="1" s="51">
       <c r="C54" s="93" t="inlineStr">
         <is>
-          <t>Root variable
-Name of variable used at the root (first) split node</t>
+          <t>Name of variable used at the root (first) split node</t>
         </is>
       </c>
       <c r="D54" s="93" t="inlineStr">
         <is>
-          <t>Root threshold ≤
-Threshold value on the left (≤) branch of the root</t>
+          <t>Threshold value on the left (≤) branch of the root</t>
         </is>
       </c>
       <c r="E54" s="93" t="inlineStr">
         <is>
-          <t>Root threshold &gt;
-Threshold value on the right (&gt;) branch of the root</t>
+          <t>Threshold value on the right (&gt;) branch of the root</t>
         </is>
       </c>
       <c r="F54" s="93" t="inlineStr">
         <is>
-          <t>Left branch – next node
-Either a leaf classification or name of second-level variable (left side)</t>
+          <t>Either a leaf classification or name of second-level variable (left side)</t>
         </is>
       </c>
       <c r="G54" s="93" t="inlineStr">
         <is>
-          <t>Left leaf – rec count
-Count of recommended foods in left leaf [ rec ]</t>
+          <t>Count of recommended foods in left leaf [ rec ]</t>
         </is>
       </c>
       <c r="H54" s="93" t="inlineStr">
         <is>
-          <t>Left leaf – not-rec count
-Count of not-recommended foods in left leaf [ not-rec ]</t>
+          <t>Count of not-recommended foods in left leaf [ not-rec ]</t>
         </is>
       </c>
       <c r="I54" s="93" t="inlineStr">
         <is>
-          <t>Right branch – next node
-Either a leaf classification or name of second-level variable (right side)</t>
+          <t>Either a leaf classification or name of second-level variable (right side)</t>
         </is>
       </c>
       <c r="J54" s="93" t="inlineStr">
         <is>
-          <t>Right leaf – rec count
-Count of recommended foods in right leaf [ rec ]</t>
+          <t>Count of recommended foods in right leaf [ rec ]</t>
         </is>
       </c>
       <c r="K54" s="93" t="inlineStr">
         <is>
-          <t>Right leaf – not-rec count
-Count of not-recommended foods in right leaf [ not-rec ]</t>
+          <t>Count of not-recommended foods in right leaf [ not-rec ]</t>
         </is>
       </c>
       <c r="L54" s="93" t="inlineStr">
         <is>
-          <t>Sub-left-left threshold/label
-Threshold or class label for sub-branch: left → left</t>
+          <t>Threshold or class label for sub-branch: left → left</t>
         </is>
       </c>
       <c r="M54" s="93" t="inlineStr">
         <is>
-          <t>Sub-left-right threshold/label
-Threshold or class label for sub-branch: left → right</t>
+          <t>Threshold or class label for sub-branch: left → right</t>
         </is>
       </c>
       <c r="N54" s="93" t="inlineStr">
         <is>
-          <t>Sub-right-left threshold/label
-Threshold or class label for sub-branch: right → left</t>
+          <t>Threshold or class label for sub-branch: right → left</t>
         </is>
       </c>
       <c r="O54" s="93" t="inlineStr">
         <is>
-          <t>Sub-right-right threshold/label
-Threshold or class label for sub-branch: right → right</t>
+          <t>Threshold or class label for sub-branch: right → right</t>
         </is>
       </c>
       <c r="P54" s="93" t="inlineStr">
         <is>
-          <t>Leaf LL – rec count
-Recommended count at leaf: left-left</t>
+          <t>Recommended count at leaf: left-left</t>
         </is>
       </c>
       <c r="Q54" s="93" t="inlineStr">
         <is>
-          <t>Leaf LL – not-rec count
-Not-recommended count at leaf: left-left</t>
+          <t>Not-recommended count at leaf: left-left</t>
         </is>
       </c>
       <c r="R54" s="93" t="inlineStr">
         <is>
-          <t>Leaf LR – rec count
-Recommended count at leaf: left-right</t>
+          <t>Recommended count at leaf: left-right</t>
         </is>
       </c>
       <c r="S54" s="93" t="inlineStr">
         <is>
-          <t>Leaf LR – not-rec count
-Not-recommended count at leaf: left-right</t>
+          <t>Not-recommended count at leaf: left-right</t>
         </is>
       </c>
       <c r="T54" s="93" t="inlineStr">
         <is>
-          <t>Leaf RL – rec count
-Recommended count at leaf: right-left</t>
+          <t>Recommended count at leaf: right-left</t>
         </is>
       </c>
       <c r="U54" s="93" t="inlineStr">
         <is>
-          <t>Leaf RL – not-rec count
-Not-recommended count at leaf: right-left</t>
+          <t>Not-recommended count at leaf: right-left</t>
         </is>
       </c>
       <c r="V54" s="93" t="inlineStr">
         <is>
-          <t>Leaf RR – rec count
-Recommended count at leaf: right-right</t>
+          <t>Recommended count at leaf: right-right</t>
         </is>
       </c>
       <c r="W54" s="93" t="inlineStr">
         <is>
-          <t>Leaf RR – not-rec count
-Not-recommended count at leaf: right-right</t>
+          <t>Not-recommended count at leaf: right-right</t>
         </is>
       </c>
     </row>
@@ -12681,20 +12553,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
       <c r="L5" s="84" t="n"/>
       <c r="M5" s="84" t="n"/>
       <c r="N5" s="84" t="n"/>
@@ -13408,20 +13276,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
       <c r="L36" s="84" t="n"/>
       <c r="M36" s="84" t="n"/>
       <c r="N36" s="84" t="n"/>
@@ -13796,62 +13660,52 @@
     <row r="54" ht="60" customHeight="1" s="51">
       <c r="C54" s="93" t="inlineStr">
         <is>
-          <t>Path A match
-Match Rule A to correct path (letter: A, B, or C)</t>
+          <t>Match Rule A to correct path (letter: A, B, or C)</t>
         </is>
       </c>
       <c r="D54" s="93" t="inlineStr">
         <is>
-          <t>Path B match
-Match Rule B to correct path (letter: A, B, or C)</t>
+          <t>Match Rule B to correct path (letter: A, B, or C)</t>
         </is>
       </c>
       <c r="E54" s="93" t="inlineStr">
         <is>
-          <t>Path C match
-Match Rule C to correct path (letter: A, B, or C)</t>
+          <t>Match Rule C to correct path (letter: A, B, or C)</t>
         </is>
       </c>
       <c r="F54" s="93" t="inlineStr">
         <is>
-          <t>Number of paths
-'My tree contains ___ paths' — total number of decision paths</t>
+          <t>'My tree contains ___ paths' — total number of decision paths</t>
         </is>
       </c>
       <c r="G54" s="93" t="inlineStr">
         <is>
-          <t>Rule 1
-Written if-then decision rule for path 1 of own tree</t>
+          <t>Written if-then decision rule for path 1 of own tree</t>
         </is>
       </c>
       <c r="H54" s="93" t="inlineStr">
         <is>
-          <t>Rule 2
-Written if-then decision rule for path 2 of own tree</t>
+          <t>Written if-then decision rule for path 2 of own tree</t>
         </is>
       </c>
       <c r="I54" s="93" t="inlineStr">
         <is>
-          <t>Rule 3
-Written if-then decision rule for path 3 of own tree</t>
+          <t>Written if-then decision rule for path 3 of own tree</t>
         </is>
       </c>
       <c r="J54" s="93" t="inlineStr">
         <is>
-          <t>Rule 4
-Written if-then decision rule for path 4 of own tree (if applicable)</t>
+          <t>Written if-then decision rule for path 4 of own tree (if applicable)</t>
         </is>
       </c>
       <c r="K54" s="93" t="inlineStr">
         <is>
-          <t>Rule 5
-Written if-then decision rule for path 5 of own tree (if applicable)</t>
+          <t>Written if-then decision rule for path 5 of own tree (if applicable)</t>
         </is>
       </c>
       <c r="L54" s="93" t="inlineStr">
         <is>
-          <t>Rule 6
-Written if-then decision rule for path 6 of own tree (if applicable)</t>
+          <t>Written if-then decision rule for path 6 of own tree (if applicable)</t>
         </is>
       </c>
     </row>
@@ -14054,16 +13908,12 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="87" t="n"/>
       <c r="H5" s="84" t="n"/>
       <c r="I5" s="84" t="n"/>
       <c r="J5" s="84" t="n"/>
@@ -14721,16 +14571,12 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="87" t="n"/>
       <c r="H36" s="84" t="n"/>
       <c r="I36" s="84" t="n"/>
       <c r="J36" s="84" t="n"/>
@@ -15077,50 +14923,42 @@
     <row r="54" ht="60" customHeight="1" s="51">
       <c r="C54" s="93" t="inlineStr">
         <is>
-          <t>Misclassification @ 28
-Number of misclassified foods if threshold = 28 kcal</t>
+          <t>Number of misclassified foods if threshold = 28 kcal</t>
         </is>
       </c>
       <c r="D54" s="93" t="inlineStr">
         <is>
-          <t>Misclassification @ 69
-Number of misclassified foods if threshold = 69 kcal</t>
+          <t>Number of misclassified foods if threshold = 69 kcal</t>
         </is>
       </c>
       <c r="E54" s="93" t="inlineStr">
         <is>
-          <t>Misclassification @ 219
-Number of misclassified foods if threshold = 219 kcal</t>
+          <t>Number of misclassified foods if threshold = 219 kcal</t>
         </is>
       </c>
       <c r="F54" s="93" t="inlineStr">
         <is>
-          <t>Misclassification @ 346
-Number of misclassified foods if threshold = 346 kcal</t>
+          <t>Number of misclassified foods if threshold = 346 kcal</t>
         </is>
       </c>
       <c r="G54" s="93" t="inlineStr">
         <is>
-          <t>Misclassification @ 359
-Number of misclassified foods if threshold = 359 kcal</t>
+          <t>Number of misclassified foods if threshold = 359 kcal</t>
         </is>
       </c>
       <c r="H54" s="93" t="inlineStr">
         <is>
-          <t>Misclassification @ 408
-Number of misclassified foods if threshold = 408 kcal</t>
+          <t>Number of misclassified foods if threshold = 408 kcal</t>
         </is>
       </c>
       <c r="I54" s="93" t="inlineStr">
         <is>
-          <t>Misclassification @ 489
-Number of misclassified foods if threshold = 489 kcal</t>
+          <t>Number of misclassified foods if threshold = 489 kcal</t>
         </is>
       </c>
       <c r="J54" s="93" t="inlineStr">
         <is>
-          <t>Optimal threshold value
-'The optimal threshold value is: ___' — threshold with fewest misclassifications</t>
+          <t>'The optimal threshold value is: ___' — threshold with fewest misclassifications</t>
         </is>
       </c>
     </row>
@@ -15479,20 +15317,16 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>Ozzy</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="n"/>
-      <c r="D5" s="84" t="n"/>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="84" t="n"/>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="84" t="n"/>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
       <c r="L5" s="84" t="n"/>
       <c r="M5" s="84" t="n"/>
       <c r="N5" s="84" t="n"/>
@@ -16536,20 +16370,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="B36" s="84" t="inlineStr">
-        <is>
-          <t>Sheila</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n"/>
-      <c r="D36" s="84" t="n"/>
-      <c r="E36" s="84" t="n"/>
-      <c r="F36" s="84" t="n"/>
-      <c r="G36" s="84" t="n"/>
-      <c r="H36" s="84" t="n"/>
-      <c r="I36" s="84" t="n"/>
-      <c r="J36" s="84" t="n"/>
-      <c r="K36" s="84" t="n"/>
+      <c r="B36" s="86" t="n"/>
+      <c r="C36" s="86" t="n"/>
+      <c r="D36" s="86" t="n"/>
+      <c r="E36" s="86" t="n"/>
+      <c r="F36" s="86" t="n"/>
+      <c r="G36" s="86" t="n"/>
+      <c r="H36" s="86" t="n"/>
+      <c r="I36" s="86" t="n"/>
+      <c r="J36" s="86" t="n"/>
+      <c r="K36" s="87" t="n"/>
       <c r="L36" s="84" t="n"/>
       <c r="M36" s="84" t="n"/>
       <c r="N36" s="84" t="n"/>
@@ -17100,128 +16930,107 @@
     <row r="54" ht="60" customHeight="1" s="51">
       <c r="C54" s="93" t="inlineStr">
         <is>
-          <t>Q4 – Can explain DT
-Yes/No: Can student explain how a decision tree works?</t>
+          <t>Yes/No: Can student explain how a decision tree works?</t>
         </is>
       </c>
       <c r="D54" s="93" t="inlineStr">
         <is>
-          <t>Q8a – Classify strawberry
-Apply the given decision tree to classify the strawberry card: 'recommended' or 'not recommended'</t>
+          <t>Apply the given decision tree to classify the strawberry card: 'recommended' or 'not recommended'</t>
         </is>
       </c>
       <c r="E54" s="93" t="inlineStr">
         <is>
-          <t>Q8b – Decision rule sentence
-Complete: 'Strawberry is classified as ___ because ___' — formulate the decision rule</t>
+          <t>Complete: 'Strawberry is classified as ___ because ___' — formulate the decision rule</t>
         </is>
       </c>
       <c r="F54" s="93" t="inlineStr">
         <is>
-          <t>Q9 – What is data?
-Open-ended (6 lines): explain what data is and why we need it</t>
+          <t>Open-ended (6 lines): explain what data is and why we need it</t>
         </is>
       </c>
       <c r="G54" s="93" t="inlineStr">
         <is>
-          <t>Q10a – DT statement 1
-True/False: DT statement a — what can a decision tree do?</t>
+          <t>True/False: DT statement a — what can a decision tree do?</t>
         </is>
       </c>
       <c r="H54" s="93" t="inlineStr">
         <is>
-          <t>Q10b – DT statement 2
-True/False: DT statement b</t>
+          <t>True/False: DT statement b</t>
         </is>
       </c>
       <c r="I54" s="93" t="inlineStr">
         <is>
-          <t>Q10c – DT statement 3
-True/False: DT statement c</t>
+          <t>True/False: DT statement c</t>
         </is>
       </c>
       <c r="J54" s="93" t="inlineStr">
         <is>
-          <t>Q10d – DT statement 4
-True/False: DT statement d</t>
+          <t>True/False: DT statement d</t>
         </is>
       </c>
       <c r="K54" s="93" t="inlineStr">
         <is>
-          <t>Q10e – DT statement 5
-True/False: DT statement e</t>
+          <t>True/False: DT statement e</t>
         </is>
       </c>
       <c r="L54" s="93" t="inlineStr">
         <is>
-          <t>Q10f – DT statement 6
-True/False: DT statement f</t>
+          <t>True/False: DT statement f</t>
         </is>
       </c>
       <c r="M54" s="93" t="inlineStr">
         <is>
-          <t>Q10g – DT statement 7
-True/False: DT statement g</t>
+          <t>True/False: DT statement g</t>
         </is>
       </c>
       <c r="N54" s="93" t="inlineStr">
         <is>
-          <t>Q10h – DT statement 8
-True/False: DT statement h</t>
+          <t>True/False: DT statement h</t>
         </is>
       </c>
       <c r="O54" s="93" t="inlineStr">
         <is>
-          <t>Q11a – Step order 1
-Rank step 1 in correct order for building a decision rule (1–4)</t>
+          <t>Rank step 1 in correct order for building a decision rule (1–4)</t>
         </is>
       </c>
       <c r="P54" s="93" t="inlineStr">
         <is>
-          <t>Q11b – Step order 2
-Rank step 2 in correct order (1–4)</t>
+          <t>Rank step 2 in correct order (1–4)</t>
         </is>
       </c>
       <c r="Q54" s="93" t="inlineStr">
         <is>
-          <t>Q11c – Step order 3
-Rank step 3 in correct order (1–4)</t>
+          <t>Rank step 3 in correct order (1–4)</t>
         </is>
       </c>
       <c r="R54" s="93" t="inlineStr">
         <is>
-          <t>Q11d – Step order 4
-Rank step 4 in correct order (1–4)</t>
+          <t>Rank step 4 in correct order (1–4)</t>
         </is>
       </c>
       <c r="S54" s="93" t="inlineStr">
         <is>
-          <t>Q12a – AI statement 1
-True/False: Why is a DT considered AI? — statement a</t>
+          <t>True/False: Why is a DT considered AI? — statement a</t>
         </is>
       </c>
       <c r="T54" s="93" t="inlineStr">
         <is>
-          <t>Q12b – AI statement 2
-True/False: AI statement b</t>
+          <t>True/False: AI statement b</t>
         </is>
       </c>
       <c r="U54" s="93" t="inlineStr">
         <is>
-          <t>Q12c – AI statement 3
-True/False: AI statement c</t>
+          <t>True/False: AI statement c</t>
         </is>
       </c>
       <c r="V54" s="93" t="inlineStr">
         <is>
-          <t>Q12d – AI statement 4
-True/False: AI statement d</t>
+          <t>True/False: AI statement d</t>
         </is>
       </c>
       <c r="W54" s="93" t="inlineStr">
         <is>
-          <t>Q12e – AI statement 5
-True/False: AI statement e</t>
+          <t>True/False: AI statement e</t>
         </is>
       </c>
     </row>

</xml_diff>